<commit_message>
Publish index.html @ 2026-10-16 10:54:46
</commit_message>
<xml_diff>
--- a/iter.xlsx
+++ b/iter.xlsx
@@ -1340,13 +1340,14 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D18"/>
+  <dimension ref="A1:E18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="56" customWidth="1" min="3" max="3"/>
-    <col width="62" customWidth="1" min="4" max="4"/>
+    <col width="52" customWidth="1" min="3" max="3"/>
+    <col width="54" customWidth="1" min="4" max="4"/>
+    <col width="58" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -1377,6 +1378,11 @@
           <t>依据（代码 / 系统现状）</t>
         </is>
       </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>缓解措施 / 影响范围</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="48" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
@@ -1399,6 +1405,11 @@
           <t>MachineAilseInfoController（售货机货道维度）；SmartAilseInfoController:216-218 售货机 / 静态柜不支持批量上新</t>
         </is>
       </c>
+      <c r="E3" s="5" t="inlineStr">
+        <is>
+          <t>已落定，无未决风险</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="76" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
@@ -1421,6 +1432,11 @@
           <t>适用机型：SmartAilseInfoController.addGoodsBatch 按「机型 source + skuId」查 getThirdSku，查不到即拒（:232-237）；建模：thirdPartySkuId 为空时抛「未绑定可售机型商品code」（AbstractSmartAisleInfoService:610-616），建模信息表 GoodsThirdPartyModelInfoMapper</t>
         </is>
       </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
+          <t>已落定，无未决风险</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="62" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
@@ -1443,6 +1459,11 @@
           <t>admin-manager-pc-2.0/…/analysis.js:133「静态柜补货单仅支持按销量生成」＝现有 PC 端前端入口约束；2026-10-16 产品裁决后 AI 卡片不沿用该约束</t>
         </is>
       </c>
+      <c r="E5" s="5" t="inlineStr">
+        <is>
+          <t>已落定，无未决风险</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="34" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
@@ -1465,8 +1486,13 @@
           <t>GoodsPriceEditorCard.vue:78-81 确认结构 { machineId, rows }，为单机改价</t>
         </is>
       </c>
-    </row>
-    <row r="7" ht="132" customHeight="1">
+      <c r="E6" s="5" t="inlineStr">
+        <is>
+          <t>已落定，无未决风险</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="160" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
           <t>5</t>
@@ -1485,6 +1511,11 @@
       <c r="D7" s="5" t="inlineStr">
         <is>
           <t>主单 ReplenishmentListMaster.java:36-76（机构维度，无 machineId）/ 子单 ReplenishmentListDetail.java:39-62（masterId+machineId+cabinetNo）；入口 ReplenishmentListMasterController.java:51-60（/service/ops/replenishment/list/master/v1/createReplenishment，返回单 Integer masterId）；实现 ReplenishmentListMasterServiceImpl.java:368-515（save master :451-452、按 machineId,cabinetNo 分组 :408-425、每组一条子单同 masterId :489-497、子单号 masterId-序号 :460）；约束 :440-449 跨多个车线路仓直接报错；ERP pick.js:10「通过单据编号获取关联机器单」</t>
+        </is>
+      </c>
+      <c r="E7" s="5" t="inlineStr">
+        <is>
+          <t>已落定，无未决风险</t>
         </is>
       </c>
     </row>
@@ -1509,8 +1540,13 @@
           <t>用户口径确认 2026-10-15；代码侧未独立复核（本机无代码库）</t>
         </is>
       </c>
-    </row>
-    <row r="9" ht="34" customHeight="1">
+      <c r="E8" s="5" t="inlineStr">
+        <is>
+          <t>已落定，无未决风险</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="48" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
           <t>7</t>
@@ -1529,6 +1565,11 @@
       <c r="D9" s="5" t="inlineStr">
         <is>
           <t>用户口径确认 2026-10-15；代码侧未独立复核</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>已落定，无未决风险</t>
         </is>
       </c>
     </row>
@@ -1553,8 +1594,13 @@
           <t>现有系统「添加商品」页（用户截图）+ 用户口径确认 2026-10-15 / 2026-10-16</t>
         </is>
       </c>
-    </row>
-    <row r="11" ht="34" customHeight="1">
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>已落定，无未决风险</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="48" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
           <t>9</t>
@@ -1575,8 +1621,13 @@
           <t>现有系统「选择机器」页（用户截图）+ 用户口径确认 2026-10-15</t>
         </is>
       </c>
-    </row>
-    <row r="12" ht="90" customHeight="1">
+      <c r="E11" s="5" t="inlineStr">
+        <is>
+          <t>已落定，无未决风险</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="104" customHeight="1">
       <c r="A12" s="4" t="inlineStr">
         <is>
           <t>10</t>
@@ -1595,6 +1646,11 @@
       <c r="D12" s="5" t="inlineStr">
         <is>
           <t>用户口径确认 2026-10-15 / 2026-10-16（现有系统「库存查询 → 生成补货单」页截图）；代码侧未独立复核</t>
+        </is>
+      </c>
+      <c r="E12" s="5" t="inlineStr">
+        <is>
+          <t>已落定，无未决风险</t>
         </is>
       </c>
     </row>
@@ -1619,6 +1675,11 @@
           <t>产品裁决 2026-10-16；与落定口径 1、2 配套</t>
         </is>
       </c>
+      <c r="E13" s="5" t="inlineStr">
+        <is>
+          <t>已落定，无未决风险</t>
+        </is>
+      </c>
     </row>
     <row r="14" ht="48" customHeight="1">
       <c r="A14" s="4" t="inlineStr">
@@ -1641,6 +1702,11 @@
           <t>产品裁决 2026-10-16；与落定口径 8 配套</t>
         </is>
       </c>
+      <c r="E14" s="5" t="inlineStr">
+        <is>
+          <t>已落定，无未决风险</t>
+        </is>
+      </c>
     </row>
     <row r="15" ht="62" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
@@ -1663,6 +1729,11 @@
           <t>产品裁决 2026-10-16</t>
         </is>
       </c>
+      <c r="E15" s="5" t="inlineStr">
+        <is>
+          <t>已落定，无未决风险</t>
+        </is>
+      </c>
     </row>
     <row r="16" ht="48" customHeight="1">
       <c r="A16" s="4" t="inlineStr">
@@ -1685,8 +1756,13 @@
           <t>产品裁决 2026-10-16</t>
         </is>
       </c>
-    </row>
-    <row r="17" ht="48" customHeight="1">
+      <c r="E16" s="5" t="inlineStr">
+        <is>
+          <t>已落定，无未决风险</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="62" customHeight="1">
       <c r="A17" s="11" t="inlineStr">
         <is>
           <t>R1</t>
@@ -1707,8 +1783,13 @@
           <t>AiChat/api.js:9-13（chat/v2 SSE 与 ca-api 交互）；cardRegistry.js:12-23（现有 10 个能力卡片）</t>
         </is>
       </c>
-    </row>
-    <row r="18" ht="34" customHeight="1">
+      <c r="E17" s="12" t="inlineStr">
+        <is>
+          <t>① 接口契约（请求 / 响应 / 错误码）随需求一并冻结，作为联调交付物；② 联调前先用 mock 契约跑通前端卡片；③ 核对不到的部分登记进 §12.2 待确认，不写进卡片文案｜影响：B7 配套能力与 mp_kb 结构无法在代码层核实</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="62" customHeight="1">
       <c r="A18" s="11" t="inlineStr">
         <is>
           <t>R2</t>
@@ -1727,6 +1808,11 @@
       <c r="D18" s="5" t="inlineStr">
         <is>
           <t>与落定口径 1、2 配套，属前端卡片与 ca-api 交互约定</t>
+        </is>
+      </c>
+      <c r="E18" s="12" t="inlineStr">
+        <is>
+          <t>① 结果卡数据模型固定为 {succ[], fail[{机器, 原因}]}，成功 + 失败 = 命中总数；② 后端按机器维度返回错误码，前端原样透传、不改写；③ 重试只对 fail 项重新签发 confirm_id｜影响：批量上下架的结果展示与重试</t>
         </is>
       </c>
     </row>
@@ -2112,14 +2198,15 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E12"/>
+  <dimension ref="A1:F12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
     <col width="22" customWidth="1" min="2" max="2"/>
     <col width="11" customWidth="1" min="3" max="3"/>
-    <col width="32" customWidth="1" min="4" max="4"/>
-    <col width="44" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="4" max="4"/>
+    <col width="38" customWidth="1" min="5" max="5"/>
+    <col width="30" customWidth="1" min="6" max="6"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -2155,6 +2242,11 @@
           <t>系统 / 代码侧依据</t>
         </is>
       </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>重新评估时机</t>
+        </is>
+      </c>
     </row>
     <row r="3" ht="48" customHeight="1">
       <c r="A3" s="14" t="inlineStr">
@@ -2182,6 +2274,11 @@
           <t>现有 MerchantOverviewCard 已覆盖今日销售额 / 订单 / 在线 / 缺货故障停售</t>
         </is>
       </c>
+      <c r="F3" s="14" t="inlineStr">
+        <is>
+          <t>—（已定处置，不再重评）</t>
+        </is>
+      </c>
     </row>
     <row r="4" ht="22" customHeight="1">
       <c r="A4" s="14" t="inlineStr">
@@ -2209,6 +2306,11 @@
           <t>引导路径与语雀《8、硬件运维》一致</t>
         </is>
       </c>
+      <c r="F4" s="14" t="inlineStr">
+        <is>
+          <t>—（已定处置，不再重评）</t>
+        </is>
+      </c>
     </row>
     <row r="5" ht="34" customHeight="1">
       <c r="A5" s="14" t="inlineStr">
@@ -2236,6 +2338,11 @@
           <t>引导路径与语雀《8、硬件运维》一致（PC 故障监控 → 故障策略配置）</t>
         </is>
       </c>
+      <c r="F5" s="14" t="inlineStr">
+        <is>
+          <t>—（已定处置，不再重评）</t>
+        </is>
+      </c>
     </row>
     <row r="6" ht="34" customHeight="1">
       <c r="A6" s="14" t="inlineStr">
@@ -2263,6 +2370,11 @@
           <t>后端校验 thirdPartySkuId（建模产物），为空即拒；建模须上传多角度图片</t>
         </is>
       </c>
+      <c r="F6" s="14" t="inlineStr">
+        <is>
+          <t>—（已定处置，不再重评）</t>
+        </is>
+      </c>
     </row>
     <row r="7" ht="22" customHeight="1">
       <c r="A7" s="14" t="inlineStr">
@@ -2290,6 +2402,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="F7" s="14" t="inlineStr">
+        <is>
+          <t>—（已定处置，不再重评）</t>
+        </is>
+      </c>
     </row>
     <row r="8" ht="22" customHeight="1">
       <c r="A8" s="14" t="inlineStr">
@@ -2317,6 +2434,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="F8" s="14" t="inlineStr">
+        <is>
+          <t>—（已定处置，不再重评）</t>
+        </is>
+      </c>
     </row>
     <row r="9" ht="22" customHeight="1">
       <c r="A9" s="14" t="inlineStr">
@@ -2344,6 +2466,11 @@
           <t>—</t>
         </is>
       </c>
+      <c r="F9" s="14" t="inlineStr">
+        <is>
+          <t>—（已定处置，不再重评）</t>
+        </is>
+      </c>
     </row>
     <row r="10" ht="22" customHeight="1">
       <c r="A10" s="14" t="inlineStr">
@@ -2371,8 +2498,13 @@
           <t>—</t>
         </is>
       </c>
-    </row>
-    <row r="11" ht="22" customHeight="1">
+      <c r="F10" s="14" t="inlineStr">
+        <is>
+          <t>—（已定处置，不再重评）</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="34" customHeight="1">
       <c r="A11" s="14" t="inlineStr">
         <is>
           <t>视频监控查看</t>
@@ -2398,8 +2530,13 @@
           <t>—</t>
         </is>
       </c>
-    </row>
-    <row r="12" ht="22" customHeight="1">
+      <c r="F11" s="14" t="inlineStr">
+        <is>
+          <t>1.2 立项评审（qa 侧若反馈答不准，提前到 1.1 收尾复评）</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="34" customHeight="1">
       <c r="A12" s="14" t="inlineStr">
         <is>
           <t>改名记录查询</t>
@@ -2423,6 +2560,11 @@
       <c r="E12" s="14" t="inlineStr">
         <is>
           <t>—</t>
+        </is>
+      </c>
+      <c r="F12" s="14" t="inlineStr">
+        <is>
+          <t>等 OS 侧提供改名操作日志数据源后复评（预计 1.2）</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Publish index.html @ 2026-10-16 11:38:50
</commit_message>
<xml_diff>
--- a/iter.xlsx
+++ b/iter.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1.1 迭代清单" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="落定口径与风险" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="系统核对与证据索引" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="不做与暂缓" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="问话依据明细" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="1.1 迭代清单" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="落定口径与风险" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="系统核对与证据索引" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="不做与暂缓" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="问话依据明细" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1065,7 +1065,7 @@
         </is>
       </c>
     </row>
-    <row r="15" ht="62" customHeight="1">
+    <row r="15" ht="90" customHeight="1">
       <c r="A15" s="4" t="inlineStr">
         <is>
           <t>C7</t>
@@ -1103,11 +1103,11 @@
       </c>
       <c r="H15" s="5" t="inlineStr">
         <is>
-          <t>支持单商品近期销售额；支持限定「所有在线机器」范围；⚠ 2026-10-16 裁决 7：卡片需给出「铺货 N 台」（该商品已铺设的机器台数），否则客户看不出铺货规模</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="34" customHeight="1">
+          <t>支持单商品近期销售额；支持限定「所有在线机器」范围；⚠ 2026-10-16 裁决 7：卡片需给出「铺货 N 台」（该商品已铺设的机器台数），否则客户看不出铺货规模；⚠ 该列需新增接口（现有接口给的是「有销售记录的机器数」，口径不同），未就绪前留空标「暂不可用」</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="104" customHeight="1">
       <c r="A16" s="4" t="inlineStr">
         <is>
           <t>C9</t>
@@ -1145,7 +1145,7 @@
       </c>
       <c r="H16" s="5" t="inlineStr">
         <is>
-          <t>由预警通知或操作日志返回离线原因；R6 仍负责给离线清单</t>
+          <t>⚠ 2026-10-16 代码复核修正：原「操作日志」来源不存在——machine_online_record 只有 online_status 等字段、无原因字段。真实来源＝monitor_fault_records（fault_type=machine_offline），建议文案＝nacos 配置（MonitorFaultRecordServiceImpl.java:130-131）。R6 仍负责给离线清单，卡片「来源」列只可能出现故障记录 / 预警通知两类</t>
         </is>
       </c>
     </row>
@@ -1384,7 +1384,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="48" customHeight="1">
+    <row r="3" ht="90" customHeight="1">
       <c r="A3" s="4" t="inlineStr">
         <is>
           <t>1</t>
@@ -1402,7 +1402,7 @@
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>MachineAilseInfoController（售货机货道维度）；SmartAilseInfoController:216-218 售货机 / 静态柜不支持批量上新</t>
+          <t>MachineAilseInfoController（售货机货道维度）；SmartAilseInfoController:216-218 售货机 / 静态柜不支持批量上新；AbstractSmartAisleInfoService:1435-1437 静态柜单机上架抛 NOT_SUPPORT_ALI_MACHINE_SHELVES。⚠ 2026-10-16 裁决：静态柜不支持上架（单机 / 批量两条路径都拦），机器选择范围排除静态柜</t>
         </is>
       </c>
       <c r="E3" s="5" t="inlineStr">
@@ -1519,7 +1519,7 @@
         </is>
       </c>
     </row>
-    <row r="8" ht="48" customHeight="1">
+    <row r="8" ht="104" customHeight="1">
       <c r="A8" s="4" t="inlineStr">
         <is>
           <t>6</t>
@@ -1532,7 +1532,7 @@
       </c>
       <c r="C8" s="5" t="inlineStr">
         <is>
-          <t>按机型分两套：智能柜＝移除该商品、库存清零；售货机＝把该货道换成默认商品（不清空，货道继续售卖）。卡片按机型出不同文案，不统一写「清空」</t>
+          <t>按机型分两套：智能柜＝移除该商品、库存清零（剔除 sku 重建货道）；售货机＝该商品所在货道停售（is_sale_enabled=N，不清空、不换商品）。⚠ 2026-10-16 代码复核修正：原「换默认商品」有误，deleteMachineGoods 售货机分支只做 updateAisleToEnable(DISABLE_AILSE)；换默认商品只发生在平台商品删除（TGoodsDeleteHandlerServiceImpl.java:174）与审核驳回两条独立路径</t>
         </is>
       </c>
       <c r="D8" s="5" t="inlineStr">
@@ -1735,7 +1735,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="48" customHeight="1">
+    <row r="16" ht="132" customHeight="1">
       <c r="A16" s="4" t="inlineStr">
         <is>
           <t>14</t>
@@ -1748,7 +1748,7 @@
       </c>
       <c r="C16" s="5" t="inlineStr">
         <is>
-          <t>2026-10-16 裁决 7：需要支持。除销量 / 销售额外给出「铺货 N 台」（该商品已铺设的机器台数），避免客户拿到销售额却判断不出铺货规模</t>
+          <t>2026-10-16 裁决 7：需要支持。除销量 / 销售额外给出「铺货 N 台」（该商品已铺设的机器台数），避免客户拿到销售额却判断不出铺货规模。⚠ 2026-10-16 代码复核：需新增接口——现有 GoodsSoldController.soldMachineNumber 取的是「有销售记录的机器数」（machine_sold_group_day_sku 的 COUNT DISTINCT machine_id），不是铺货数；铺货口径在 GoodsSoldMapper.xml:280+（GoodsDisplay 服务），Controller 未暴露。接口未就绪前该列留空标「暂不可用」，不得用卖过的机器数顶替</t>
         </is>
       </c>
       <c r="D16" s="5" t="inlineStr">
@@ -2102,7 +2102,7 @@
     <row r="22" ht="34" customHeight="1">
       <c r="A22" s="5" t="inlineStr">
         <is>
-          <t>旧约束：静态柜前端仅提供「按销量」入口</t>
+          <t>旧约束：静态柜前端仅提供「按销量」入口（另一条独立约束：静态柜不支持上下架，见证据索引）</t>
         </is>
       </c>
       <c r="B22" s="5" t="inlineStr">
@@ -2159,7 +2159,7 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="34" customHeight="1">
+    <row r="27" ht="62" customHeight="1">
       <c r="A27" s="5" t="inlineStr">
         <is>
           <t>支付方式记录</t>
@@ -2167,7 +2167,7 @@
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>micro-service-data/…/OfflinePayRecordController.java、RptDayReceivePaymentController.java</t>
+          <t>micro-service-data/…/OfflinePayRecordController.java（拆现金内部纸币 / 硬币 pay_type 1/2）、RptDayReceivePaymentController.java（拆 app_id / machine_type / type）——⚠ 两者都不是「支付渠道」维度，2026-10-16 裁决后 R4 按微信 / 支付宝 / 现金 / 刷卡等渠道拆分，数据源须另行确认</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Publish index.html @ 2026-10-16 12:03:55
</commit_message>
<xml_diff>
--- a/iter.xlsx
+++ b/iter.xlsx
@@ -1023,7 +1023,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="34" customHeight="1">
+    <row r="14" ht="76" customHeight="1">
       <c r="A14" s="4" t="inlineStr">
         <is>
           <t>C4</t>
@@ -1051,7 +1051,7 @@
       </c>
       <c r="F14" s="5" t="inlineStr">
         <is>
-          <t>现金多少，打卡多少。分别是多少</t>
+          <t>现金多少，刷卡多少。分别是多少（口语「打卡」＝「刷卡」，见配套 B7 归一化）</t>
         </is>
       </c>
       <c r="G14" s="5" t="inlineStr">
@@ -1061,7 +1061,7 @@
       </c>
       <c r="H14" s="5" t="inlineStr">
         <is>
-          <t>默认给合计，用户要求时按支付方式拆分展示</t>
+          <t>默认给合计，用户要求时按支付方式拆分展示。⚠ 拆分维度＝微信 / 支付宝 / 现金 / 刷卡等渠道；现金＝现金支付总额，不拆纸币 / 硬币（取 OfflinePayRecordController 的 pay_type 1/2 合计）。刷卡若取不到数则降级为微信 / 支付宝 / 现金三类</t>
         </is>
       </c>
     </row>
@@ -1107,7 +1107,7 @@
         </is>
       </c>
     </row>
-    <row r="16" ht="104" customHeight="1">
+    <row r="16" ht="132" customHeight="1">
       <c r="A16" s="4" t="inlineStr">
         <is>
           <t>C9</t>
@@ -1140,16 +1140,16 @@
       </c>
       <c r="G16" s="5" t="inlineStr">
         <is>
-          <t>MachineOnlineRecordDataController、MonitorFaultRecordController（micro-service-data）</t>
+          <t>MonitorFaultRecordController（micro-service-data，monitor_fault_records · fault_type=machine_offline）；MachineOnlineRecordDataController（仅上下线状态，无原因字段，不能作来源）</t>
         </is>
       </c>
       <c r="H16" s="5" t="inlineStr">
         <is>
-          <t>⚠ 2026-10-16 代码复核修正：原「操作日志」来源不存在——machine_online_record 只有 online_status 等字段、无原因字段。真实来源＝monitor_fault_records（fault_type=machine_offline），建议文案＝nacos 配置（MonitorFaultRecordServiceImpl.java:130-131）。R6 仍负责给离线清单，卡片「来源」列只可能出现故障记录 / 预警通知两类</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="34" customHeight="1">
+          <t>⚠ 2026-10-16 代码复核修正：原「操作日志」来源不存在——machine_online_record 只有 online_status 等字段、无原因字段。真实来源＝monitor_fault_records（fault_type=machine_offline），建议文案＝nacos 配置（MonitorFaultRecordServiceImpl.java:130-131）。R6 仍负责给离线清单。⚠ 2026-10-16 第二轮收口：「预警通知」同样未核（无表/接口证据），本期不采用，卡片「来源」列只写「故障记录」，预警通知转需求说明 §12.2 第 10 条待确认</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="90" customHeight="1">
       <c r="A17" s="4" t="inlineStr">
         <is>
           <t>B7</t>
@@ -1177,7 +1177,7 @@
       </c>
       <c r="F17" s="5" t="inlineStr">
         <is>
-          <t>缺货↔空货、离线↔「高线」、营业额↔实收；纯点位名/编号开场 ×61</t>
+          <t>缺货↔空货、离线↔「高线」、营业额↔实收；纯点位名/编号开场 ×61；⚠ 2026-10-16 补：支付渠道口语归一化「打卡」↔「刷卡」（源问法「现金多少，打卡多少」，打卡＝刷卡/银行卡，非考勤打卡）</t>
         </is>
       </c>
       <c r="G17" s="5" t="inlineStr">
@@ -1492,7 +1492,7 @@
         </is>
       </c>
     </row>
-    <row r="7" ht="160" customHeight="1">
+    <row r="7" ht="188" customHeight="1">
       <c r="A7" s="4" t="inlineStr">
         <is>
           <t>5</t>
@@ -1510,7 +1510,7 @@
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>主单 ReplenishmentListMaster.java:36-76（机构维度，无 machineId）/ 子单 ReplenishmentListDetail.java:39-62（masterId+machineId+cabinetNo）；入口 ReplenishmentListMasterController.java:51-60（/service/ops/replenishment/list/master/v1/createReplenishment，返回单 Integer masterId）；实现 ReplenishmentListMasterServiceImpl.java:368-515（save master :451-452、按 machineId,cabinetNo 分组 :408-425、每组一条子单同 masterId :489-497、子单号 masterId-序号 :460）；约束 :440-449 跨多个车线路仓直接报错；ERP pick.js:10「通过单据编号获取关联机器单」</t>
+          <t>主单 ReplenishmentListMaster.java:36-76（机构维度，无 machineId）/ 子单 ReplenishmentListDetail.java:39-62（masterId+machineId+cabinetNo）；入口 ReplenishmentListMasterController.java:51-60（/service/ops/replenishment/list/master/v1/createReplenishment，返回单 Integer masterId）；实现 ReplenishmentListMasterServiceImpl.java:368-515（save master :451-452、按 machineId,cabinetNo 分组 :408-425、每组一条子单同 masterId :489-497、子单号 masterId-序号 :460）；约束 :439-449 跨多个车线路仓直接报错，⚠ 但该校验外层包了 ispReplenishSku 开关，仅启用 ISP 服务商补货时生效；普通运营商跨仓不报错（合成一张主单），AI 须在提交前按仓分组提示；ERP pick.js:10「通过单据编号获取关联机器单」</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr">
@@ -1537,7 +1537,7 @@
       </c>
       <c r="D8" s="5" t="inlineStr">
         <is>
-          <t>用户口径确认 2026-10-15；代码侧未独立复核（本机无代码库）</t>
+          <t>用户口径确认 2026-10-15；✅ 2026-10-16 代码侧已独立复核并修正：MachineAisleInfoServiceImpl.deleteMachineGoods:2527-2541 售货机分支＝updateAisleToEnable(DISABLE_AILSE)，仅 set is_sale_enabled=N；:2542 起智能柜分支＝剔除 sku 重建货道+库存清零。原「换默认商品」口径已废</t>
         </is>
       </c>
       <c r="E8" s="5" t="inlineStr">
@@ -1546,7 +1546,7 @@
         </is>
       </c>
     </row>
-    <row r="9" ht="48" customHeight="1">
+    <row r="9" ht="104" customHeight="1">
       <c r="A9" s="4" t="inlineStr">
         <is>
           <t>7</t>
@@ -1564,7 +1564,7 @@
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>用户口径确认 2026-10-15；代码侧未独立复核</t>
+          <t>用户口径确认 2026-10-15；✅ 2026-10-16 代码侧已独立复核：最大库存无独立配置表，即 machine_aisle_info.default_goods_stock（MachineAisleInfo.defaultGoodsStock）；补货量 diffStock＝默认库存−现有库存。⚠ 须取 micro-service-analysis 真实字段，禁用 micro-service-data 旧实现的 goodsStock*2 硬编码（ReplenishmentDataServiceImpl.java:646）</t>
         </is>
       </c>
       <c r="E9" s="5" t="inlineStr">
@@ -1645,7 +1645,7 @@
       </c>
       <c r="D12" s="5" t="inlineStr">
         <is>
-          <t>用户口径确认 2026-10-15 / 2026-10-16（现有系统「库存查询 → 生成补货单」页截图）；代码侧未独立复核</t>
+          <t>用户口径确认 2026-10-15 / 2026-10-16；依据为业务方提供的「添加商品」页截图，**页面形态本身**未经代码复核（本机无代码库）。⚠ 注意区分：本表其余涉及后端逻辑的条目已于 2026-10-16 完成代码侧复核并标注 ✅，本条「未复核」仅指前端页面截图依据，不代表整体未核</t>
         </is>
       </c>
       <c r="E12" s="5" t="inlineStr">
@@ -2962,7 +2962,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="22" customHeight="1">
+    <row r="20" ht="34" customHeight="1">
       <c r="A20" s="5" t="inlineStr">
         <is>
           <t>C4 支付方式</t>
@@ -2970,7 +2970,7 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>现金多少，打卡多少。分别是多少</t>
+          <t>现金多少，刷卡多少。分别是多少（口语「打卡」＝「刷卡」）</t>
         </is>
       </c>
       <c r="C20" s="4" t="n">
@@ -2978,7 +2978,7 @@
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>1.1 R11：按需拆分支付方式</t>
+          <t>1.1 R11：按需拆分支付方式；现金＝现金支付总额，不拆纸币 / 硬币</t>
         </is>
       </c>
     </row>
@@ -3062,7 +3062,7 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="22" customHeight="1">
+    <row r="25" ht="104" customHeight="1">
       <c r="A25" s="5" t="inlineStr">
         <is>
           <t>C9 离线原因</t>
@@ -3078,7 +3078,7 @@
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>数据源：预警通知 / 操作日志</t>
+          <t>数据源：monitor_fault_records 故障记录表（fault_type=machine_offline），建议文案＝nacos 配置。⚠ 2026-10-16 复核：「操作日志」来源不存在（machine_online_record 无原因字段）；「预警通知」同样未核，本期不采用，转入需求说明 §12.2 第 10 条</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Publish index.html @ 2026-10-16 14:33:20
</commit_message>
<xml_diff>
--- a/iter.xlsx
+++ b/iter.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="1.1 迭代清单" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="落定口径与风险" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="系统核对与证据索引" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="不做与暂缓" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="问话依据明细" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1.1 迭代清单" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="落定口径与风险" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="系统核对与证据索引" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="不做与暂缓" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="问话依据明细" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1023,7 +1023,7 @@
         </is>
       </c>
     </row>
-    <row r="14" ht="76" customHeight="1">
+    <row r="14" ht="90" customHeight="1">
       <c r="A14" s="4" t="inlineStr">
         <is>
           <t>C4</t>
@@ -1056,12 +1056,12 @@
       </c>
       <c r="G14" s="5" t="inlineStr">
         <is>
-          <t>OfflinePayRecordController、RptDayReceivePaymentController（data / ops）</t>
+          <t>machine_sold_group_day_new（getMachinesSoldSumGroupByDayNew，MachineSoldGroupDayService.java:122），支付方式名经 provide_pay_type.payName 映射。⚠ 已排除 OfflinePayRecordController / RptDayReceivePaymentController（非支付渠道维度）</t>
         </is>
       </c>
       <c r="H14" s="5" t="inlineStr">
         <is>
-          <t>默认给合计，用户要求时按支付方式拆分展示。⚠ 拆分维度＝微信 / 支付宝 / 现金 / 刷卡等渠道；现金＝现金支付总额，不拆纸币 / 硬币（取 OfflinePayRecordController 的 pay_type 1/2 合计）。刷卡若取不到数则降级为微信 / 支付宝 / 现金三类</t>
+          <t>默认给合计，用户要求时按支付方式拆分展示。⚠ 2026-10-16 定稿：动态枚举——只列统计期内产生过销售额的支付方式，不写死渠道清单；现金＝现金支付总额，不拆纸币 / 硬币；刷卡＝真实存在的支付方式（MachineSoldProfitBO.cardTotalAmount），不需要降级方案</t>
         </is>
       </c>
     </row>
@@ -1145,7 +1145,7 @@
       </c>
       <c r="H16" s="5" t="inlineStr">
         <is>
-          <t>⚠ 2026-10-16 代码复核修正：原「操作日志」来源不存在——machine_online_record 只有 online_status 等字段、无原因字段。真实来源＝monitor_fault_records（fault_type=machine_offline），建议文案＝nacos 配置（MonitorFaultRecordServiceImpl.java:130-131）。R6 仍负责给离线清单。⚠ 2026-10-16 第二轮收口：「预警通知」同样未核（无表/接口证据），本期不采用，卡片「来源」列只写「故障记录」，预警通知转需求说明 §12.2 第 10 条待确认</t>
+          <t>⚠ 2026-10-16 代码复核修正：原「操作日志」来源不存在——machine_online_record 只有 online_status 等字段、无原因字段。真实来源＝monitor_fault_records（fault_type=machine_offline），建议文案＝nacos 配置（MonitorFaultRecordServiceImpl.java:130-131）。R6 仍负责给离线清单。⚠ 2026-10-16 第二轮收口：「预警通知」同样未核（无表/接口证据），本期不采用，卡片「来源」列只写「故障记录」，预警通知转需求说明 §12.2 第 4 条待确认</t>
         </is>
       </c>
     </row>
@@ -2159,15 +2159,15 @@
         </is>
       </c>
     </row>
-    <row r="27" ht="62" customHeight="1">
+    <row r="27" ht="76" customHeight="1">
       <c r="A27" s="5" t="inlineStr">
         <is>
-          <t>支付方式记录</t>
+          <t>支付方式记录（R4 数据源）</t>
         </is>
       </c>
       <c r="B27" s="5" t="inlineStr">
         <is>
-          <t>micro-service-data/…/OfflinePayRecordController.java（拆现金内部纸币 / 硬币 pay_type 1/2）、RptDayReceivePaymentController.java（拆 app_id / machine_type / type）——⚠ 两者都不是「支付渠道」维度，2026-10-16 裁决后 R4 按微信 / 支付宝 / 现金 / 刷卡等渠道拆分，数据源须另行确认</t>
+          <t>micro-service-analysis/…/MachineSoldGroupDayService.java:122 getMachinesSoldSumGroupByDayNew（`machine_sold_group_day_new`，方法注释「各支付方式收入」），支付方式名经 provide_pay_type.payName 映射。⚠ 已排除 micro-service-data/…/OfflinePayRecordController.java（拆现金内部纸币 / 硬币 pay_type 1/2）与 RptDayReceivePaymentController.java（拆 app_id / machine_type / type）——两者都不是「支付渠道」维度</t>
         </is>
       </c>
     </row>
@@ -3078,7 +3078,7 @@
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>数据源：monitor_fault_records 故障记录表（fault_type=machine_offline），建议文案＝nacos 配置。⚠ 2026-10-16 复核：「操作日志」来源不存在（machine_online_record 无原因字段）；「预警通知」同样未核，本期不采用，转入需求说明 §12.2 第 10 条</t>
+          <t>数据源：monitor_fault_records 故障记录表（fault_type=machine_offline），建议文案＝nacos 配置。⚠ 2026-10-16 复核：「操作日志」来源不存在（machine_online_record 无原因字段）；「预警通知」同样未核，本期不采用，转入需求说明 §12.2 第 4 条</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Publish index.html @ 2026-10-16 16:14:04
</commit_message>
<xml_diff>
--- a/iter.xlsx
+++ b/iter.xlsx
@@ -1340,7 +1340,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E18"/>
+  <dimension ref="A1:E20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1573,7 +1573,7 @@
         </is>
       </c>
     </row>
-    <row r="10" ht="76" customHeight="1">
+    <row r="10" ht="132" customHeight="1">
       <c r="A10" s="4" t="inlineStr">
         <is>
           <t>8</t>
@@ -1586,7 +1586,7 @@
       </c>
       <c r="C10" s="5" t="inlineStr">
         <is>
-          <t>沿用现有「添加商品」页骨架：私有商品库选择，仅展示当前机型可售商品；价格默认带出商品库自身价且可改。⚠ 2026-10-16 裁决 5：多机型批量上架时按「本批机器机型的交集」过滤（单台＝该机机型）；弹层内须写明过滤范围并点名被滤掉的商品，不让用户以为数据丢了</t>
+          <t>沿用现有「添加商品」页骨架：私有商品库选择，仅展示当前机型可售商品；价格默认带出商品库自身价且可改。⚠ 2026-10-16 裁决 5：多机型批量上架时按「本批机器机型的交集」过滤（单台＝该机机型）；弹层内须写明过滤范围并点名被滤掉的商品，不让用户以为数据丢了。⚠ PC 端（2026-10-16）＝居中弹窗对齐现有系统；⚠ 校验前移·商品级：商品在本机 / 本批机器上未绑定可售机型商品 code 时直接置灰标「⛔ 不可上架：原因」、不可加入（2026-10-16 产品反馈）</t>
         </is>
       </c>
       <c r="D10" s="5" t="inlineStr">
@@ -1600,7 +1600,7 @@
         </is>
       </c>
     </row>
-    <row r="11" ht="48" customHeight="1">
+    <row r="11" ht="118" customHeight="1">
       <c r="A11" s="4" t="inlineStr">
         <is>
           <t>9</t>
@@ -1613,12 +1613,12 @@
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>沿用现有「选择机器」页骨架：行内展示机器编号 + 名称 + 地址全称（地址完整展示、可换行不省略），不展示图片</t>
+          <t>沿用现有「选择机器」页骨架：行内展示机器编号 + 名称 + 地址全称（地址完整展示、可换行不省略），不展示图片。⚠ PC 端（2026-10-16）＝居中弹窗对齐现有系统（筛选 / 表格 / 分页 / 已选计数，勾选跨页保留）；⚠ 校验前移·机型级：不支持上架的机器直接置灰标「⛔ 不可上架：不支持在该机型售卖」、不可勾选、不进全选（2026-10-16 产品反馈：这种校验不应该在选择机器的时候就直接校验吗）</t>
         </is>
       </c>
       <c r="D11" s="5" t="inlineStr">
         <is>
-          <t>现有系统「选择机器」页（用户截图）+ 用户口径确认 2026-10-15</t>
+          <t>现有系统「选择机器」页（用户截图）+ 用户口径确认 2026-10-15 / 2026-10-16</t>
         </is>
       </c>
       <c r="E11" s="5" t="inlineStr">
@@ -1762,55 +1762,109 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="62" customHeight="1">
-      <c r="A17" s="11" t="inlineStr">
+    <row r="17" ht="118" customHeight="1">
+      <c r="A17" s="4" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>选择阶段校验前移（P1 / P2 / W6）</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-16 产品反馈：机型 / 建模类校验在**选择阶段**就挡掉，不要等执行后才报错——① P2 选择机器弹层：不支持上架的机器（如格子柜）直接置灰、标「⛔ 不可上架：不支持在该机型售卖」、checkbox 禁用、不进全选；② P1 添加商品弹层：商品在本机 / 本批机器上未绑定可售机型商品 code 时置灰标原因、不可加入。执行层 W6 结果卡逐台透传原因**保留作兜底**（「全部机器 / 按线路」范围仍可能带入不支持机器）</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>产品反馈 2026-10-16（附批量上架结果卡失败截图）；与落定口径 1、2、12 配套</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr">
+        <is>
+          <t>已落定，无未决风险</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="76" customHeight="1">
+      <c r="A18" s="4" t="inlineStr">
+        <is>
+          <t>16</t>
+        </is>
+      </c>
+      <c r="B18" s="5" t="inlineStr">
+        <is>
+          <t>上架卡补货量默认值（W1 / W2）</t>
+        </is>
+      </c>
+      <c r="C18" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-16 产品确认：默认补货量＝商品**箱规 × 1.5**（四舍五入取整），添加商品后带出、可逐项手改；**箱规为 0 或未配置 → 补货量与箱规列都展示 0**，不做其他兜底。⚠ 与 W5 补货单口径区分：补货单补货量＝最大库存 − 现存（落定口径 3），两卡口径不同</t>
+        </is>
+      </c>
+      <c r="D18" s="5" t="inlineStr">
+        <is>
+          <t>产品反馈 2026-10-16（参照现有系统「添加商品后补货数带值」截图）</t>
+        </is>
+      </c>
+      <c r="E18" s="5" t="inlineStr">
+        <is>
+          <t>已落定，无未决风险</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="62" customHeight="1">
+      <c r="A19" s="11" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
-      <c r="B17" s="12" t="inlineStr">
+      <c r="B19" s="12" t="inlineStr">
         <is>
           <t>ca-api 不在代码库（盲区）</t>
         </is>
       </c>
-      <c r="C17" s="5" t="inlineStr">
+      <c r="C19" s="5" t="inlineStr">
         <is>
           <t>B7（NLU 泛化 + 机器点名 / 上下文）与 mp_kb 知识库结构无法在代码层面核对，只能核对到数据源与前端卡片缺口；需 ca-api 侧另行确认</t>
         </is>
       </c>
-      <c r="D17" s="5" t="inlineStr">
+      <c r="D19" s="5" t="inlineStr">
         <is>
           <t>AiChat/api.js:9-13（chat/v2 SSE 与 ca-api 交互）；cardRegistry.js:12-23（现有 10 个能力卡片）</t>
         </is>
       </c>
-      <c r="E17" s="12" t="inlineStr">
+      <c r="E19" s="12" t="inlineStr">
         <is>
           <t>① 接口契约（请求 / 响应 / 错误码）随需求一并冻结，作为联调交付物；② 联调前先用 mock 契约跑通前端卡片；③ 核对不到的部分登记进 §12.2 待确认，不写进卡片文案｜影响：B7 配套能力与 mp_kb 结构无法在代码层核实</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="62" customHeight="1">
-      <c r="A18" s="11" t="inlineStr">
+    <row r="20" ht="62" customHeight="1">
+      <c r="A20" s="11" t="inlineStr">
         <is>
           <t>R2</t>
         </is>
       </c>
-      <c r="B18" s="12" t="inlineStr">
+      <c r="B20" s="12" t="inlineStr">
         <is>
           <t>多台循环上架的部分失败反馈</t>
         </is>
       </c>
-      <c r="C18" s="5" t="inlineStr">
+      <c r="C20" s="5" t="inlineStr">
         <is>
           <t>单机循环时若部分机器被后台校验拦截（不支持机型 / 未绑定商品 code），需逐台列出失败机器与原因，不得整批报失败</t>
         </is>
       </c>
-      <c r="D18" s="5" t="inlineStr">
+      <c r="D20" s="5" t="inlineStr">
         <is>
           <t>与落定口径 1、2 配套，属前端卡片与 ca-api 交互约定</t>
         </is>
       </c>
-      <c r="E18" s="12" t="inlineStr">
+      <c r="E20" s="12" t="inlineStr">
         <is>
           <t>① 结果卡数据模型固定为 {succ[], fail[{机器, 原因}]}，成功 + 失败 = 命中总数；② 后端按机器维度返回错误码，前端原样透传、不改写；③ 重试只对 fail 项重新签发 confirm_id｜影响：批量上下架的结果展示与重试</t>
         </is>

</xml_diff>

<commit_message>
Publish index.html @ 2026-10-16 16:38:03
</commit_message>
<xml_diff>
--- a/iter.xlsx
+++ b/iter.xlsx
@@ -1340,7 +1340,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E20"/>
+  <dimension ref="A1:E21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1816,55 +1816,82 @@
         </is>
       </c>
     </row>
-    <row r="19" ht="62" customHeight="1">
-      <c r="A19" s="11" t="inlineStr">
-        <is>
-          <t>R1</t>
-        </is>
-      </c>
-      <c r="B19" s="12" t="inlineStr">
-        <is>
-          <t>ca-api 不在代码库（盲区）</t>
+    <row r="19" ht="132" customHeight="1">
+      <c r="A19" s="4" t="inlineStr">
+        <is>
+          <t>17</t>
+        </is>
+      </c>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>订单明细两段式：先选单后看明细（R2 / B3）</t>
         </is>
       </c>
       <c r="C19" s="5" t="inlineStr">
         <is>
-          <t>B7（NLU 泛化 + 机器点名 / 上下文）与 mp_kb 知识库结构无法在代码层面核对，只能核对到数据源与前端卡片缺口；需 ca-api 侧另行确认</t>
+          <t>2026-10-16 产品反馈：泛问「查订单明细」时不应直接甩一单的明细——AI **先反问「要查哪一单」**并给**最近订单选择列表**（最近 5 单 · 近 7 天 · 按时间倒序；行＝订单号 / 机器 / 商品 / 金额 / 支付 / 状态，行可点，附「可直接发订单号」提示），点单才展开该单商品明细；明细态给「‹ 返回订单列表」可切回重选。**点名订单号或说「此单 / 这笔」→ 跳过选择直接出明细**。接口对应 order_recent（列表）+ order_detail（按单号）</t>
         </is>
       </c>
       <c r="D19" s="5" t="inlineStr">
         <is>
-          <t>AiChat/api.js:9-13（chat/v2 SSE 与 ca-api 交互）；cardRegistry.js:12-23（现有 10 个能力卡片）</t>
-        </is>
-      </c>
-      <c r="E19" s="12" t="inlineStr">
-        <is>
-          <t>① 接口契约（请求 / 响应 / 错误码）随需求一并冻结，作为联调交付物；② 联调前先用 mock 契约跑通前端卡片；③ 核对不到的部分登记进 §12.2 待确认，不写进卡片文案｜影响：B7 配套能力与 mp_kb 结构无法在代码层核实</t>
+          <t>产品反馈 2026-10-16（附原型「直接甩单条明细」截图）</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr">
+        <is>
+          <t>已落定，无未决风险</t>
         </is>
       </c>
     </row>
     <row r="20" ht="62" customHeight="1">
       <c r="A20" s="11" t="inlineStr">
         <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="B20" s="12" t="inlineStr">
+        <is>
+          <t>ca-api 不在代码库（盲区）</t>
+        </is>
+      </c>
+      <c r="C20" s="5" t="inlineStr">
+        <is>
+          <t>B7（NLU 泛化 + 机器点名 / 上下文）与 mp_kb 知识库结构无法在代码层面核对，只能核对到数据源与前端卡片缺口；需 ca-api 侧另行确认</t>
+        </is>
+      </c>
+      <c r="D20" s="5" t="inlineStr">
+        <is>
+          <t>AiChat/api.js:9-13（chat/v2 SSE 与 ca-api 交互）；cardRegistry.js:12-23（现有 10 个能力卡片）</t>
+        </is>
+      </c>
+      <c r="E20" s="12" t="inlineStr">
+        <is>
+          <t>① 接口契约（请求 / 响应 / 错误码）随需求一并冻结，作为联调交付物；② 联调前先用 mock 契约跑通前端卡片；③ 核对不到的部分登记进 §12.2 待确认，不写进卡片文案｜影响：B7 配套能力与 mp_kb 结构无法在代码层核实</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="62" customHeight="1">
+      <c r="A21" s="11" t="inlineStr">
+        <is>
           <t>R2</t>
         </is>
       </c>
-      <c r="B20" s="12" t="inlineStr">
+      <c r="B21" s="12" t="inlineStr">
         <is>
           <t>多台循环上架的部分失败反馈</t>
         </is>
       </c>
-      <c r="C20" s="5" t="inlineStr">
+      <c r="C21" s="5" t="inlineStr">
         <is>
           <t>单机循环时若部分机器被后台校验拦截（不支持机型 / 未绑定商品 code），需逐台列出失败机器与原因，不得整批报失败</t>
         </is>
       </c>
-      <c r="D20" s="5" t="inlineStr">
+      <c r="D21" s="5" t="inlineStr">
         <is>
           <t>与落定口径 1、2 配套，属前端卡片与 ca-api 交互约定</t>
         </is>
       </c>
-      <c r="E20" s="12" t="inlineStr">
+      <c r="E21" s="12" t="inlineStr">
         <is>
           <t>① 结果卡数据模型固定为 {succ[], fail[{机器, 原因}]}，成功 + 失败 = 命中总数；② 后端按机器维度返回错误码，前端原样透传、不改写；③ 重试只对 fail 项重新签发 confirm_id｜影响：批量上下架的结果展示与重试</t>
         </is>

</xml_diff>

<commit_message>
Publish index.html @ 2026-10-19 10:10:51
</commit_message>
<xml_diff>
--- a/iter.xlsx
+++ b/iter.xlsx
@@ -1340,7 +1340,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E21"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1843,55 +1843,82 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="62" customHeight="1">
-      <c r="A20" s="11" t="inlineStr">
-        <is>
-          <t>R1</t>
-        </is>
-      </c>
-      <c r="B20" s="12" t="inlineStr">
-        <is>
-          <t>ca-api 不在代码库（盲区）</t>
+    <row r="20" ht="104" customHeight="1">
+      <c r="A20" s="4" t="inlineStr">
+        <is>
+          <t>18</t>
+        </is>
+      </c>
+      <c r="B20" s="5" t="inlineStr">
+        <is>
+          <t>W2-b 线路选择＝真下拉（W2-b / A1）</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>B7（NLU 泛化 + 机器点名 / 上下文）与 mp_kb 知识库结构无法在代码层面核对，只能核对到数据源与前端卡片缺口；需 ca-api 侧另行确认</t>
+          <t>2026-10-19 产品反馈：「点一下切换线路，我不能直接选定要切换到那条线路」——kv「线路」行改为**真下拉**：点开列出该商户下**全部线路机构**（每行＝线路名 + 台数，当前线路高亮 ✓），**点选哪条就切到哪条**（不是点击循环切到下一条）；点卡片外任意处收起；diff 区提示「点线路名可下拉切换」。需求说明 §12.1 定稿 #10</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>AiChat/api.js:9-13（chat/v2 SSE 与 ca-api 交互）；cardRegistry.js:12-23（现有 10 个能力卡片）</t>
-        </is>
-      </c>
-      <c r="E20" s="12" t="inlineStr">
-        <is>
-          <t>① 接口契约（请求 / 响应 / 错误码）随需求一并冻结，作为联调交付物；② 联调前先用 mock 契约跑通前端卡片；③ 核对不到的部分登记进 §12.2 待确认，不写进卡片文案｜影响：B7 配套能力与 mp_kb 结构无法在代码层核实</t>
+          <t>产品反馈 2026-10-19（附 PC 端原型截图）；设计稿 / 承载形态表此前已写「下拉」但原型实现为循环切换，本次对齐</t>
+        </is>
+      </c>
+      <c r="E20" s="5" t="inlineStr">
+        <is>
+          <t>已落定，无未决风险</t>
         </is>
       </c>
     </row>
     <row r="21" ht="62" customHeight="1">
       <c r="A21" s="11" t="inlineStr">
         <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="B21" s="12" t="inlineStr">
+        <is>
+          <t>ca-api 不在代码库（盲区）</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>B7（NLU 泛化 + 机器点名 / 上下文）与 mp_kb 知识库结构无法在代码层面核对，只能核对到数据源与前端卡片缺口；需 ca-api 侧另行确认</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>AiChat/api.js:9-13（chat/v2 SSE 与 ca-api 交互）；cardRegistry.js:12-23（现有 10 个能力卡片）</t>
+        </is>
+      </c>
+      <c r="E21" s="12" t="inlineStr">
+        <is>
+          <t>① 接口契约（请求 / 响应 / 错误码）随需求一并冻结，作为联调交付物；② 联调前先用 mock 契约跑通前端卡片；③ 核对不到的部分登记进 §12.2 待确认，不写进卡片文案｜影响：B7 配套能力与 mp_kb 结构无法在代码层核实</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="62" customHeight="1">
+      <c r="A22" s="11" t="inlineStr">
+        <is>
           <t>R2</t>
         </is>
       </c>
-      <c r="B21" s="12" t="inlineStr">
+      <c r="B22" s="12" t="inlineStr">
         <is>
           <t>多台循环上架的部分失败反馈</t>
         </is>
       </c>
-      <c r="C21" s="5" t="inlineStr">
+      <c r="C22" s="5" t="inlineStr">
         <is>
           <t>单机循环时若部分机器被后台校验拦截（不支持机型 / 未绑定商品 code），需逐台列出失败机器与原因，不得整批报失败</t>
         </is>
       </c>
-      <c r="D21" s="5" t="inlineStr">
+      <c r="D22" s="5" t="inlineStr">
         <is>
           <t>与落定口径 1、2 配套，属前端卡片与 ca-api 交互约定</t>
         </is>
       </c>
-      <c r="E21" s="12" t="inlineStr">
+      <c r="E22" s="12" t="inlineStr">
         <is>
           <t>① 结果卡数据模型固定为 {succ[], fail[{机器, 原因}]}，成功 + 失败 = 命中总数；② 后端按机器维度返回错误码，前端原样透传、不改写；③ 重试只对 fail 项重新签发 confirm_id｜影响：批量上下架的结果展示与重试</t>
         </is>

</xml_diff>

<commit_message>
Publish index.html @ 2026-10-19 10:42:59
</commit_message>
<xml_diff>
--- a/iter.xlsx
+++ b/iter.xlsx
@@ -1843,7 +1843,7 @@
         </is>
       </c>
     </row>
-    <row r="20" ht="104" customHeight="1">
+    <row r="20" ht="118" customHeight="1">
       <c r="A20" s="4" t="inlineStr">
         <is>
           <t>18</t>
@@ -1851,17 +1851,17 @@
       </c>
       <c r="B20" s="5" t="inlineStr">
         <is>
-          <t>W2-b 线路选择＝真下拉（W2-b / A1）</t>
+          <t>W2-b 线路选择＝点选直接切换，两端形态不同（W2-b / A1）</t>
         </is>
       </c>
       <c r="C20" s="5" t="inlineStr">
         <is>
-          <t>2026-10-19 产品反馈：「点一下切换线路，我不能直接选定要切换到那条线路」——kv「线路」行改为**真下拉**：点开列出该商户下**全部线路机构**（每行＝线路名 + 台数，当前线路高亮 ✓），**点选哪条就切到哪条**（不是点击循环切到下一条）；点卡片外任意处收起；diff 区提示「点线路名可下拉切换」。需求说明 §12.1 定稿 #10</t>
+          <t>2026-10-19 产品反馈：「点一下切换线路，我不能直接选定要切换到那条线路」——点「线路」行列出该商户下**全部线路机构**（线路名 + 台数，当前线路高亮 ✓），**点选哪条就切到哪条**（不是点击循环切到下一条）。两端形态：**移动端＝底部半屏弹层**（同 P1 / P2 选择形态——移动端选择类交互无「卡内嵌下拉」先例，追问「移动端有这种交互吗」后改）；**PC 端＝卡内真下拉**（点卡片外收起）。需求说明 §12.1 定稿 #10</t>
         </is>
       </c>
       <c r="D20" s="5" t="inlineStr">
         <is>
-          <t>产品反馈 2026-10-19（附 PC 端原型截图）；设计稿 / 承载形态表此前已写「下拉」但原型实现为循环切换，本次对齐</t>
+          <t>产品反馈 2026-10-19（附两端原型截图）；设计稿 / 承载形态表此前已写「下拉」但原型实现为循环切换，本次对齐</t>
         </is>
       </c>
       <c r="E20" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Publish index.html @ 2026-10-21 11:03:26
</commit_message>
<xml_diff>
--- a/iter.xlsx
+++ b/iter.xlsx
@@ -1340,7 +1340,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E22"/>
+  <dimension ref="A1:E23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1870,55 +1870,82 @@
         </is>
       </c>
     </row>
-    <row r="21" ht="62" customHeight="1">
-      <c r="A21" s="11" t="inlineStr">
-        <is>
-          <t>R1</t>
-        </is>
-      </c>
-      <c r="B21" s="12" t="inlineStr">
-        <is>
-          <t>ca-api 不在代码库（盲区）</t>
+    <row r="21" ht="272" customHeight="1">
+      <c r="A21" s="4" t="inlineStr">
+        <is>
+          <t>19</t>
+        </is>
+      </c>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>知识问答补缺口 + 「去操作」入口（KB 补丁层 / 定稿 #11）</t>
         </is>
       </c>
       <c r="C21" s="5" t="inlineStr">
         <is>
-          <t>B7（NLU 泛化 + 机器点名 / 上下文）与 mp_kb 知识库结构无法在代码层面核对，只能核对到数据源与前端卡片缺口；需 ca-api 侧另行确认</t>
+          <t>2026-10-21 覆盖率实测（654 条真实问话逐条喂路由，非静态对照）：命中 467/654＝71.4%。补四处：① **新增条目「新增商品（商品库入库）」**——「怎么新增商品」出现 **44 次**，此前写能力不接 + KB 不命中＝双落空；② 已有条目补口语同义词：设备注册（怎么注册机器 5 次）/ 库存盘点（库存账实不符 2 次）/ 温度设置（怎么控制温度 1 次）；③ 只读护栏补口语词「那些 / 那几台 / 有那」，并规定**清单句式 + 缺货 → 先给缺货清单**（「那些在线的机器缺货百分之四十以上」要的是缺货清单，不是在线机器清单）；④ **知识答案底部「去操作」入口**：只有答案讲的是某后台页面上的操作才挂（本期＝去新增商品），一行＝动作名 + 路径，点击＝跳转对应页面，**AI 不代填、不发写操作**。⚠ KB 改动全部走**补丁层叠加**（KB11_ENTRIES / KB11_ALIAS / resolveKB11），**不动 1.0 源自动生成的 KB 区块**；补同义词**不加过长 key**（实测「怎么注册一台机器」会被 LCS 用「一台机器」匹配「有一台机器离线了」得 0.45，越过 0.42 阈值误答成设备注册）。补完 → 523/654＝80.0%</t>
         </is>
       </c>
       <c r="D21" s="5" t="inlineStr">
         <is>
-          <t>AiChat/api.js:9-13（chat/v2 SSE 与 ca-api 交互）；cardRegistry.js:12-23（现有 10 个能力卡片）</t>
-        </is>
-      </c>
-      <c r="E21" s="12" t="inlineStr">
-        <is>
-          <t>① 接口契约（请求 / 响应 / 错误码）随需求一并冻结，作为联调交付物；② 联调前先用 mock 契约跑通前端卡片；③ 核对不到的部分登记进 §12.2 待确认，不写进卡片文案｜影响：B7 配套能力与 mp_kb 结构无法在代码层核实</t>
+          <t>覆盖率实测 654 条 + 产品裁决 2026-10-21（「走知识库回答，然后支持点击跳转至对应的新增商品页面」）；需求说明 §4.2 / §4.5 / §12.1 定稿 #11；卡片设计稿 K1</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr">
+        <is>
+          <t>已落定，无未决风险</t>
         </is>
       </c>
     </row>
     <row r="22" ht="62" customHeight="1">
       <c r="A22" s="11" t="inlineStr">
         <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="B22" s="12" t="inlineStr">
+        <is>
+          <t>ca-api 不在代码库（盲区）</t>
+        </is>
+      </c>
+      <c r="C22" s="5" t="inlineStr">
+        <is>
+          <t>B7（NLU 泛化 + 机器点名 / 上下文）与 mp_kb 知识库结构无法在代码层面核对，只能核对到数据源与前端卡片缺口；需 ca-api 侧另行确认</t>
+        </is>
+      </c>
+      <c r="D22" s="5" t="inlineStr">
+        <is>
+          <t>AiChat/api.js:9-13（chat/v2 SSE 与 ca-api 交互）；cardRegistry.js:12-23（现有 10 个能力卡片）</t>
+        </is>
+      </c>
+      <c r="E22" s="12" t="inlineStr">
+        <is>
+          <t>① 接口契约（请求 / 响应 / 错误码）随需求一并冻结，作为联调交付物；② 联调前先用 mock 契约跑通前端卡片；③ 核对不到的部分登记进 §12.2 待确认，不写进卡片文案｜影响：B7 配套能力与 mp_kb 结构无法在代码层核实</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="62" customHeight="1">
+      <c r="A23" s="11" t="inlineStr">
+        <is>
           <t>R2</t>
         </is>
       </c>
-      <c r="B22" s="12" t="inlineStr">
+      <c r="B23" s="12" t="inlineStr">
         <is>
           <t>多台循环上架的部分失败反馈</t>
         </is>
       </c>
-      <c r="C22" s="5" t="inlineStr">
+      <c r="C23" s="5" t="inlineStr">
         <is>
           <t>单机循环时若部分机器被后台校验拦截（不支持机型 / 未绑定商品 code），需逐台列出失败机器与原因，不得整批报失败</t>
         </is>
       </c>
-      <c r="D22" s="5" t="inlineStr">
+      <c r="D23" s="5" t="inlineStr">
         <is>
           <t>与落定口径 1、2 配套，属前端卡片与 ca-api 交互约定</t>
         </is>
       </c>
-      <c r="E22" s="12" t="inlineStr">
+      <c r="E23" s="12" t="inlineStr">
         <is>
           <t>① 结果卡数据模型固定为 {succ[], fail[{机器, 原因}]}，成功 + 失败 = 命中总数；② 后端按机器维度返回错误码，前端原样透传、不改写；③ 重试只对 fail 项重新签发 confirm_id｜影响：批量上下架的结果展示与重试</t>
         </is>

</xml_diff>

<commit_message>
Publish index.html @ 2026-10-22 10:39:50
</commit_message>
<xml_diff>
--- a/iter.xlsx
+++ b/iter.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1.1 迭代清单" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="落定口径与风险" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="系统核对与证据索引" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="不做与暂缓" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="问话依据明细" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="1.1 迭代清单" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="落定口径与风险" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="系统核对与证据索引" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="不做与暂缓" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="问话依据明细" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1340,7 +1340,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1897,55 +1897,82 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="62" customHeight="1">
-      <c r="A22" s="11" t="inlineStr">
-        <is>
-          <t>R1</t>
-        </is>
-      </c>
-      <c r="B22" s="12" t="inlineStr">
-        <is>
-          <t>ca-api 不在代码库（盲区）</t>
+    <row r="22" ht="188" customHeight="1">
+      <c r="A22" s="4" t="inlineStr">
+        <is>
+          <t>20</t>
+        </is>
+      </c>
+      <c r="B22" s="5" t="inlineStr">
+        <is>
+          <t>原型交互修正四项（定稿 #12）</t>
         </is>
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>B7（NLU 泛化 + 机器点名 / 上下文）与 mp_kb 知识库结构无法在代码层面核对，只能核对到数据源与前端卡片缺口；需 ca-api 侧另行确认</t>
+          <t>2026-10-22 产品反馈（附 4 张原型截图）：① **W3 下架卡「添加机器」只列已铺该商品的机器**——sheetAddMachine / modalAddMachine 增加 pname 参数，按下架商品过滤，没铺货的机器不进弹层（没铺货无从下架）；② **经营只读解析时间范围**——bizAsk 解析「最近 / 近 N 天 · N 天内 · 本月 / 这个月 / 当月」，sales / orders 卡按区间出数（标题「近 30 天」/「本月」，接口 range=30d / month），不再一律答今日；③ **W1 上架卡 diff 区标题直接叫「价格改动」**、逐行列改价商品与改前 → 改后，无改动整块不展示（原「将上架 N 项」标题撤下，件数由按钮承担）；④ **补货单逻辑复核**——确认现行＝按库存生成（补货量＝最大库存 − 现存，定稿 #4 口径不变），仅复核不改版</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>AiChat/api.js:9-13（chat/v2 SSE 与 ca-api 交互）；cardRegistry.js:12-23（现有 10 个能力卡片）</t>
-        </is>
-      </c>
-      <c r="E22" s="12" t="inlineStr">
-        <is>
-          <t>① 接口契约（请求 / 响应 / 错误码）随需求一并冻结，作为联调交付物；② 联调前先用 mock 契约跑通前端卡片；③ 核对不到的部分登记进 §12.2 待确认，不写进卡片文案｜影响：B7 配套能力与 mp_kb 结构无法在代码层核实</t>
+          <t>产品反馈 2026-10-22（附原型截图 4 张）；需求说明 §4.1 / §5.1 / §5.3 / §7.2 / §12.1 定稿 #12；冒烟 MP 133 / PC 155</t>
+        </is>
+      </c>
+      <c r="E22" s="5" t="inlineStr">
+        <is>
+          <t>已落定，无未决风险</t>
         </is>
       </c>
     </row>
     <row r="23" ht="62" customHeight="1">
       <c r="A23" s="11" t="inlineStr">
         <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="B23" s="12" t="inlineStr">
+        <is>
+          <t>ca-api 不在代码库（盲区）</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>B7（NLU 泛化 + 机器点名 / 上下文）与 mp_kb 知识库结构无法在代码层面核对，只能核对到数据源与前端卡片缺口；需 ca-api 侧另行确认</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>AiChat/api.js:9-13（chat/v2 SSE 与 ca-api 交互）；cardRegistry.js:12-23（现有 10 个能力卡片）</t>
+        </is>
+      </c>
+      <c r="E23" s="12" t="inlineStr">
+        <is>
+          <t>① 接口契约（请求 / 响应 / 错误码）随需求一并冻结，作为联调交付物；② 联调前先用 mock 契约跑通前端卡片；③ 核对不到的部分登记进 §12.2 待确认，不写进卡片文案｜影响：B7 配套能力与 mp_kb 结构无法在代码层核实</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="62" customHeight="1">
+      <c r="A24" s="11" t="inlineStr">
+        <is>
           <t>R2</t>
         </is>
       </c>
-      <c r="B23" s="12" t="inlineStr">
+      <c r="B24" s="12" t="inlineStr">
         <is>
           <t>多台循环上架的部分失败反馈</t>
         </is>
       </c>
-      <c r="C23" s="5" t="inlineStr">
+      <c r="C24" s="5" t="inlineStr">
         <is>
           <t>单机循环时若部分机器被后台校验拦截（不支持机型 / 未绑定商品 code），需逐台列出失败机器与原因，不得整批报失败</t>
         </is>
       </c>
-      <c r="D23" s="5" t="inlineStr">
+      <c r="D24" s="5" t="inlineStr">
         <is>
           <t>与落定口径 1、2 配套，属前端卡片与 ca-api 交互约定</t>
         </is>
       </c>
-      <c r="E23" s="12" t="inlineStr">
+      <c r="E24" s="12" t="inlineStr">
         <is>
           <t>① 结果卡数据模型固定为 {succ[], fail[{机器, 原因}]}，成功 + 失败 = 命中总数；② 后端按机器维度返回错误码，前端原样透传、不改写；③ 重试只对 fail 项重新签发 confirm_id｜影响：批量上下架的结果展示与重试</t>
         </is>

</xml_diff>

<commit_message>
Publish index.html @ 2026-10-22 11:12:58
</commit_message>
<xml_diff>
--- a/iter.xlsx
+++ b/iter.xlsx
@@ -1897,7 +1897,7 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="188" customHeight="1">
+    <row r="22" ht="286" customHeight="1">
       <c r="A22" s="4" t="inlineStr">
         <is>
           <t>20</t>
@@ -1910,12 +1910,12 @@
       </c>
       <c r="C22" s="5" t="inlineStr">
         <is>
-          <t>2026-10-22 产品反馈（附 4 张原型截图）：① **W3 下架卡「添加机器」只列已铺该商品的机器**——sheetAddMachine / modalAddMachine 增加 pname 参数，按下架商品过滤，没铺货的机器不进弹层（没铺货无从下架）；② **经营只读解析时间范围**——bizAsk 解析「最近 / 近 N 天 · N 天内 · 本月 / 这个月 / 当月」，sales / orders 卡按区间出数（标题「近 30 天」/「本月」，接口 range=30d / month），不再一律答今日；③ **W1 上架卡 diff 区标题直接叫「价格改动」**、逐行列改价商品与改前 → 改后，无改动整块不展示（原「将上架 N 项」标题撤下，件数由按钮承担）；④ **补货单逻辑复核**——确认现行＝按库存生成（补货量＝最大库存 − 现存，定稿 #4 口径不变），仅复核不改版</t>
+          <t>2026-10-22 产品反馈（附 4 张原型截图）：① **W3 下架卡「添加机器」只列已铺该商品的机器**——sheetAddMachine / modalAddMachine 增加 pname 参数，按下架商品过滤，没铺货的机器不进弹层（没铺货无从下架）；② **经营只读解析时间范围**——bizAsk 解析「最近 / 近 N 天 · N 天内 · 本月 / 这个月 / 当月」，sales / orders 卡按区间出数（标题「近 30 天」/「本月」，接口 range=30d / month），不再一律答今日；③ **W1 上架卡 diff 区标题直接叫「价格改动」**、逐行列改价商品与改前 → 改后，无改动整块不展示（原「将上架 N 项」标题撤下，件数由按钮承担）；④ **补货单逻辑复核**——确认现行＝按库存生成（补货量＝最大库存 − 现存，定稿 #4 口径不变），仅复核不改版；⑤ **开场槽位期点 1.1 快捷问法不再被反问机器**——1.0 版 looksLikeOtherIntent 白名单缺「上架 / 下架 / 铺货」，开场挂着等机器名的上下文时点下架 chip 被反问「没认出机器」；app3 后置覆盖该函数补白名单 + 知识命中出口接 KB 补丁层。⚠ 冒烟盲区：jsdom 载入后 guideStart 未执行、ctx 为 null，恰好绕开此路径——已补带上下文的真实开场流断言（MP 137 / PC 157）</t>
         </is>
       </c>
       <c r="D22" s="5" t="inlineStr">
         <is>
-          <t>产品反馈 2026-10-22（附原型截图 4 张）；需求说明 §4.1 / §5.1 / §5.3 / §7.2 / §12.1 定稿 #12；冒烟 MP 133 / PC 155</t>
+          <t>产品反馈 2026-10-22（附原型截图）；需求说明 §4.1 / §4.4 / §5.1 / §5.3 / §7.2 / §12.1 定稿 #12；冒烟 MP 137 / PC 157</t>
         </is>
       </c>
       <c r="E22" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Publish index.html @ 2026-10-22 11:49:12
</commit_message>
<xml_diff>
--- a/iter.xlsx
+++ b/iter.xlsx
@@ -1,17 +1,17 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="1.1 迭代清单" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="落定口径与风险" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="系统核对与证据索引" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="不做与暂缓" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="问话依据明细" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1.1 迭代清单" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="落定口径与风险" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="系统核对与证据索引" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="不做与暂缓" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="问话依据明细" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -1340,7 +1340,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1924,55 +1924,82 @@
         </is>
       </c>
     </row>
-    <row r="23" ht="62" customHeight="1">
-      <c r="A23" s="11" t="inlineStr">
-        <is>
-          <t>R1</t>
-        </is>
-      </c>
-      <c r="B23" s="12" t="inlineStr">
-        <is>
-          <t>ca-api 不在代码库（盲区）</t>
+    <row r="23" ht="286" customHeight="1">
+      <c r="A23" s="4" t="inlineStr">
+        <is>
+          <t>21</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>原型交互修正两项（定稿 #13）</t>
         </is>
       </c>
       <c r="C23" s="5" t="inlineStr">
         <is>
-          <t>B7（NLU 泛化 + 机器点名 / 上下文）与 mp_kb 知识库结构无法在代码层面核对，只能核对到数据源与前端卡片缺口；需 ca-api 侧另行确认</t>
+          <t>2026-10-22 产品反馈（附 2 张原型截图）：① **上架卡位置选择给真弹层**——「第 2 层 ▾ / A3 货道 ▾」原来只弹 toast，改呼出选择弹层（新增 slotOptions / sheetPickSlot / modalPickSlot / bindSlotPicker）：列出该机器**全部层 / 货道**并标注状态（已铺标「已有：商品名」，售货机再带「· 最大 N · 现存 M」；未铺标「空闲」），**点选即回填 chip**，售货机副行「最大 · 现存」联动刷新；移动端＝底部半屏弹层、PC 端＝居中弹窗，与既有 P1 / P2 选择形态一致；② **下架卡预览给真实价格与库存**——预览**只列还在售该商品的机器**（智能柜已移除 / 售货机货道已停售的不再列出），逐台读出该商品在这台机器上的真实现价与现有库存，**缺失值不用 0 顶替**（不再出现「¥0.00 · 库存 0」空行）；部分机器被过滤时执行说明行写明「已跳过 N 台未铺该商品的机器」；**命中 0 台走空状态卡**（标题「没有可下架的机器」），且**空状态分支必须返回卡片容器**——返回 null 会让路由以为没命中意图、掉进兜底话术「暂时无法回答」；配套修正下架执行**不再改写商品名**（原「…（货道停售）」改名会让后续按原名的检索落空，是 0/0 空行的根因之一）</t>
         </is>
       </c>
       <c r="D23" s="5" t="inlineStr">
         <is>
-          <t>AiChat/api.js:9-13（chat/v2 SSE 与 ca-api 交互）；cardRegistry.js:12-23（现有 10 个能力卡片）</t>
-        </is>
-      </c>
-      <c r="E23" s="12" t="inlineStr">
-        <is>
-          <t>① 接口契约（请求 / 响应 / 错误码）随需求一并冻结，作为联调交付物；② 联调前先用 mock 契约跑通前端卡片；③ 核对不到的部分登记进 §12.2 待确认，不写进卡片文案｜影响：B7 配套能力与 mp_kb 结构无法在代码层核实</t>
+          <t>产品反馈 2026-10-22（附原型截图）；需求说明 §5.1 / §5.3 / §8 原则 11 / §12.1 定稿 #13；卡片设计稿 W1 / W1-b / W3；冒烟 MP 141 / PC 161</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr">
+        <is>
+          <t>已落定，无未决风险</t>
         </is>
       </c>
     </row>
     <row r="24" ht="62" customHeight="1">
       <c r="A24" s="11" t="inlineStr">
         <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="B24" s="12" t="inlineStr">
+        <is>
+          <t>ca-api 不在代码库（盲区）</t>
+        </is>
+      </c>
+      <c r="C24" s="5" t="inlineStr">
+        <is>
+          <t>B7（NLU 泛化 + 机器点名 / 上下文）与 mp_kb 知识库结构无法在代码层面核对，只能核对到数据源与前端卡片缺口；需 ca-api 侧另行确认</t>
+        </is>
+      </c>
+      <c r="D24" s="5" t="inlineStr">
+        <is>
+          <t>AiChat/api.js:9-13（chat/v2 SSE 与 ca-api 交互）；cardRegistry.js:12-23（现有 10 个能力卡片）</t>
+        </is>
+      </c>
+      <c r="E24" s="12" t="inlineStr">
+        <is>
+          <t>① 接口契约（请求 / 响应 / 错误码）随需求一并冻结，作为联调交付物；② 联调前先用 mock 契约跑通前端卡片；③ 核对不到的部分登记进 §12.2 待确认，不写进卡片文案｜影响：B7 配套能力与 mp_kb 结构无法在代码层核实</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="62" customHeight="1">
+      <c r="A25" s="11" t="inlineStr">
+        <is>
           <t>R2</t>
         </is>
       </c>
-      <c r="B24" s="12" t="inlineStr">
+      <c r="B25" s="12" t="inlineStr">
         <is>
           <t>多台循环上架的部分失败反馈</t>
         </is>
       </c>
-      <c r="C24" s="5" t="inlineStr">
+      <c r="C25" s="5" t="inlineStr">
         <is>
           <t>单机循环时若部分机器被后台校验拦截（不支持机型 / 未绑定商品 code），需逐台列出失败机器与原因，不得整批报失败</t>
         </is>
       </c>
-      <c r="D24" s="5" t="inlineStr">
+      <c r="D25" s="5" t="inlineStr">
         <is>
           <t>与落定口径 1、2 配套，属前端卡片与 ca-api 交互约定</t>
         </is>
       </c>
-      <c r="E24" s="12" t="inlineStr">
+      <c r="E25" s="12" t="inlineStr">
         <is>
           <t>① 结果卡数据模型固定为 {succ[], fail[{机器, 原因}]}，成功 + 失败 = 命中总数；② 后端按机器维度返回错误码，前端原样透传、不改写；③ 重试只对 fail 项重新签发 confirm_id｜影响：批量上下架的结果展示与重试</t>
         </is>

</xml_diff>

<commit_message>
Publish index.html @ 2026-10-22 13:46:41
</commit_message>
<xml_diff>
--- a/iter.xlsx
+++ b/iter.xlsx
@@ -1340,7 +1340,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E25"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1951,55 +1951,82 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="62" customHeight="1">
-      <c r="A24" s="11" t="inlineStr">
-        <is>
-          <t>R1</t>
-        </is>
-      </c>
-      <c r="B24" s="12" t="inlineStr">
-        <is>
-          <t>ca-api 不在代码库（盲区）</t>
+    <row r="24" ht="202" customHeight="1">
+      <c r="A24" s="4" t="inlineStr">
+        <is>
+          <t>22</t>
+        </is>
+      </c>
+      <c r="B24" s="5" t="inlineStr">
+        <is>
+          <t>智能柜层容量口径（定稿 #14）</t>
         </is>
       </c>
       <c r="C24" s="5" t="inlineStr">
         <is>
-          <t>B7（NLU 泛化 + 机器点名 / 上下文）与 mp_kb 知识库结构无法在代码层面核对，只能核对到数据源与前端卡片缺口；需 ca-api 侧另行确认</t>
+          <t>2026-10-22 产品反馈（附 2 张原型截图：售货机货道展示没问题；智能柜「一层标已有商品」会误导）：**一层没有可上架商品数的限制**，限制只有机器总上架数＝**层数 × 10**（一层可能放十几个商品）。落地：① `slotOptions` 按层聚合多商品（`by` 改数组），`slotRowTxt` 对智能柜把该层已放商品逐个列出（「已有：A、B」）——「已有」**不构成占用，选已有商品的层合法并正常回填**；售货机一货道一商品，保留「已有：」＋「· 最大 N · 现存 M」占用语义；② 智能柜场景弹层必须带口径说明「智能柜一层可放多个商品 · 机器总上架数上限＝层数 × 10」（移动端＝列表上方一行，PC 端＝弹窗底部 `.pm-selcnt` 说明位），**售货机场景不出现这句**；③ 卡内机型行「无货道，按层」同步带「一层可放多个商品」</t>
         </is>
       </c>
       <c r="D24" s="5" t="inlineStr">
         <is>
-          <t>AiChat/api.js:9-13（chat/v2 SSE 与 ca-api 交互）；cardRegistry.js:12-23（现有 10 个能力卡片）</t>
-        </is>
-      </c>
-      <c r="E24" s="12" t="inlineStr">
-        <is>
-          <t>① 接口契约（请求 / 响应 / 错误码）随需求一并冻结，作为联调交付物；② 联调前先用 mock 契约跑通前端卡片；③ 核对不到的部分登记进 §12.2 待确认，不写进卡片文案｜影响：B7 配套能力与 mp_kb 结构无法在代码层核实</t>
+          <t>产品反馈 2026-10-22（附原型截图）；需求说明 §5.1 / §12.1 定稿 #14；卡片设计稿 W1 / W1-b；冒烟 MP 144 / PC 162（含「售货机弹层不带容量说明」反向断言）</t>
+        </is>
+      </c>
+      <c r="E24" s="5" t="inlineStr">
+        <is>
+          <t>已落定，无未决风险</t>
         </is>
       </c>
     </row>
     <row r="25" ht="62" customHeight="1">
       <c r="A25" s="11" t="inlineStr">
         <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="B25" s="12" t="inlineStr">
+        <is>
+          <t>ca-api 不在代码库（盲区）</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>B7（NLU 泛化 + 机器点名 / 上下文）与 mp_kb 知识库结构无法在代码层面核对，只能核对到数据源与前端卡片缺口；需 ca-api 侧另行确认</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>AiChat/api.js:9-13（chat/v2 SSE 与 ca-api 交互）；cardRegistry.js:12-23（现有 10 个能力卡片）</t>
+        </is>
+      </c>
+      <c r="E25" s="12" t="inlineStr">
+        <is>
+          <t>① 接口契约（请求 / 响应 / 错误码）随需求一并冻结，作为联调交付物；② 联调前先用 mock 契约跑通前端卡片；③ 核对不到的部分登记进 §12.2 待确认，不写进卡片文案｜影响：B7 配套能力与 mp_kb 结构无法在代码层核实</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="62" customHeight="1">
+      <c r="A26" s="11" t="inlineStr">
+        <is>
           <t>R2</t>
         </is>
       </c>
-      <c r="B25" s="12" t="inlineStr">
+      <c r="B26" s="12" t="inlineStr">
         <is>
           <t>多台循环上架的部分失败反馈</t>
         </is>
       </c>
-      <c r="C25" s="5" t="inlineStr">
+      <c r="C26" s="5" t="inlineStr">
         <is>
           <t>单机循环时若部分机器被后台校验拦截（不支持机型 / 未绑定商品 code），需逐台列出失败机器与原因，不得整批报失败</t>
         </is>
       </c>
-      <c r="D25" s="5" t="inlineStr">
+      <c r="D26" s="5" t="inlineStr">
         <is>
           <t>与落定口径 1、2 配套，属前端卡片与 ca-api 交互约定</t>
         </is>
       </c>
-      <c r="E25" s="12" t="inlineStr">
+      <c r="E26" s="12" t="inlineStr">
         <is>
           <t>① 结果卡数据模型固定为 {succ[], fail[{机器, 原因}]}，成功 + 失败 = 命中总数；② 后端按机器维度返回错误码，前端原样透传、不改写；③ 重试只对 fail 项重新签发 confirm_id｜影响：批量上下架的结果展示与重试</t>
         </is>

</xml_diff>

<commit_message>
Publish 1.1 prototypes @ 2026-10-28 14:50 (BUILD 20261028b · 定稿 #16 补货单先选机器 + 机器编号)
</commit_message>
<xml_diff>
--- a/iter.xlsx
+++ b/iter.xlsx
@@ -687,7 +687,7 @@
         </is>
       </c>
     </row>
-    <row r="6" ht="132" customHeight="1">
+    <row r="6" ht="230" customHeight="1">
       <c r="A6" s="4" t="inlineStr">
         <is>
           <t>B2</t>
@@ -725,7 +725,7 @@
       </c>
       <c r="H6" s="5" t="inlineStr">
         <is>
-          <t>单台 / 多台都做；多台合并生成【一张主单 + 每台一条子单】，禁止逐台循环调用（会出多张主单）；跨车线路仓需按仓分开提交。⚠ 2026-10-16 裁决 6：不做系统建议量，补货量一律＝最大库存（后台「补满」配置值）− 现存，不调销量算法，原「按销量 / 按补满库存」二选一取消、卡片不再有模式切换。手机端列＝商品 / 缺货数 / 缺货箱数 / 补货量（不显示价格与商品 ID）；PC 端再把「现存 / 最大库存 / 箱规」提为独立列</t>
+          <t>单台 / 多台都做；多台合并生成【一张主单 + 每台一条子单】，禁止逐台循环调用（会出多张主单）；跨车线路仓需按仓分开提交。⚠ 2026-10-16 裁决 6：不做系统建议量，补货量一律＝最大库存（后台「补满」配置值）− 现存，不调销量算法，原「按销量 / 按补满库存」二选一取消、卡片不再有模式切换。手机端列＝商品 / 缺货数 / 缺货箱数 / 补货量（不显示价格与商品 ID）；PC 端再把「现存 / 最大库存 / 箱规」提为独立列。⚠ 2026-10-28 定稿 16：机器范围不由 AI 代选——未点名机器先出「选择补货机器」卡（缺货率倒序，逐台给编号 / 名称 / 缺货率 / 状态，默认勾中 ≥30% 且可补的机器，停售 / 故障默认不勾，0 台走空状态卡），勾选后才进 W5；点名机器直接出卡。W5 卡内新增「补货机器明细」块（逐台 编号 · 名称 · 缺货率，默认展开可收起）；底部 100-1 / 100-2 是子单号、不替代机器编号</t>
         </is>
       </c>
     </row>
@@ -1340,7 +1340,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -1978,55 +1978,82 @@
         </is>
       </c>
     </row>
-    <row r="25" ht="62" customHeight="1">
-      <c r="A25" s="11" t="inlineStr">
-        <is>
-          <t>R1</t>
-        </is>
-      </c>
-      <c r="B25" s="12" t="inlineStr">
-        <is>
-          <t>ca-api 不在代码库（盲区）</t>
+    <row r="25" ht="286" customHeight="1">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>23</t>
+        </is>
+      </c>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>补货单机器范围与机器编号（W5 / B2 · 定稿 #16）</t>
         </is>
       </c>
       <c r="C25" s="5" t="inlineStr">
         <is>
-          <t>B7（NLU 泛化 + 机器点名 / 上下文）与 mp_kb 知识库结构无法在代码层面核对，只能核对到数据源与前端卡片缺口；需 ca-api 侧另行确认</t>
+          <t>2026-10-28 产品反馈（原话「我输入补货单为什么就直接给我三台缺货机器了，不应该是让我选择机器吗？还有就是这样批量生成补货单的时候为什么没有具体的机器编号」）：**机器范围不由 AI 默认代选**。① 未点名机器（「生成补货单」/ 技能清单点「补货单」）→ 先出「选择补货机器」卡：候选＝当前缺货机器，按缺货率倒序，逐台给 编号 / 名称 / 缺货率 / 状态；默认勾中缺货率 ≥30% 且可补的机器；**已停售 / 故障中的机器默认不勾**（机器本身不卖货，补了也用不上），**离线不影响**（补货是线下动作，人到了照样能补）；候选 0 台走空状态卡，不生成补货单、不给空表与确认按钮。② 已点名机器（「给欢乐颂 5 号机生成补货单」）→ 跳过选择直接出 W5，与上架「点名机器直接出卡」一致。③ W5 卡内新增「补货机器明细」块，逐台给 机器编号 / 名称 / 缺货率，**默认展开**、机器多时可收起——确认前必须能核对给哪几台补。⚠ 原实现问题：`cardReplenish` 兜底硬编码 `['hls','lj3','nwhh']` 三台演示机器，路由层同样兜底，冒烟还钉着「直接出卡」，故每次回归都通过；机器编号只以**子单号**形式出现在「生成结构」说明区（100-1 / 100-2），不是机器编号</t>
         </is>
       </c>
       <c r="D25" s="5" t="inlineStr">
         <is>
-          <t>AiChat/api.js:9-13（chat/v2 SSE 与 ca-api 交互）；cardRegistry.js:12-23（现有 10 个能力卡片）</t>
-        </is>
-      </c>
-      <c r="E25" s="12" t="inlineStr">
-        <is>
-          <t>① 接口契约（请求 / 响应 / 错误码）随需求一并冻结，作为联调交付物；② 联调前先用 mock 契约跑通前端卡片；③ 核对不到的部分登记进 §12.2 待确认，不写进卡片文案｜影响：B7 配套能力与 mp_kb 结构无法在代码层核实</t>
+          <t>产品反馈 2026-10-28（附原型截图）；需求说明 §5.5 / §12.1 定稿 #16；卡片设计稿 W5；冒烟 MP 156 / PC 169（新增 MP +12 / PC +7，含「选择卡不是确认卡」「机器明细默认展开」断言）</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="inlineStr">
+        <is>
+          <t>已落定，无未决风险</t>
         </is>
       </c>
     </row>
     <row r="26" ht="62" customHeight="1">
       <c r="A26" s="11" t="inlineStr">
         <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="B26" s="12" t="inlineStr">
+        <is>
+          <t>ca-api 不在代码库（盲区）</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>B7（NLU 泛化 + 机器点名 / 上下文）与 mp_kb 知识库结构无法在代码层面核对，只能核对到数据源与前端卡片缺口；需 ca-api 侧另行确认</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>AiChat/api.js:9-13（chat/v2 SSE 与 ca-api 交互）；cardRegistry.js:12-23（现有 10 个能力卡片）</t>
+        </is>
+      </c>
+      <c r="E26" s="12" t="inlineStr">
+        <is>
+          <t>① 接口契约（请求 / 响应 / 错误码）随需求一并冻结，作为联调交付物；② 联调前先用 mock 契约跑通前端卡片；③ 核对不到的部分登记进 §12.2 待确认，不写进卡片文案｜影响：B7 配套能力与 mp_kb 结构无法在代码层核实</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="62" customHeight="1">
+      <c r="A27" s="11" t="inlineStr">
+        <is>
           <t>R2</t>
         </is>
       </c>
-      <c r="B26" s="12" t="inlineStr">
+      <c r="B27" s="12" t="inlineStr">
         <is>
           <t>多台循环上架的部分失败反馈</t>
         </is>
       </c>
-      <c r="C26" s="5" t="inlineStr">
+      <c r="C27" s="5" t="inlineStr">
         <is>
           <t>单机循环时若部分机器被后台校验拦截（不支持机型 / 未绑定商品 code），需逐台列出失败机器与原因，不得整批报失败</t>
         </is>
       </c>
-      <c r="D26" s="5" t="inlineStr">
+      <c r="D27" s="5" t="inlineStr">
         <is>
           <t>与落定口径 1、2 配套，属前端卡片与 ca-api 交互约定</t>
         </is>
       </c>
-      <c r="E26" s="12" t="inlineStr">
+      <c r="E27" s="12" t="inlineStr">
         <is>
           <t>① 结果卡数据模型固定为 {succ[], fail[{机器, 原因}]}，成功 + 失败 = 命中总数；② 后端按机器维度返回错误码，前端原样透传、不改写；③ 重试只对 fail 项重新签发 confirm_id｜影响：批量上下架的结果展示与重试</t>
         </is>

</xml_diff>

<commit_message>
Publish index.html @ 2026-10-28 17:26:44
</commit_message>
<xml_diff>
--- a/iter.xlsx
+++ b/iter.xlsx
@@ -603,7 +603,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="104" customHeight="1">
+    <row r="4" ht="244" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
           <t>A1</t>
@@ -616,7 +616,7 @@
       </c>
       <c r="C4" s="5" t="inlineStr">
         <is>
-          <t>W1 / W1-b / W2-a·b·c / W6 / W6-b</t>
+          <t>W1 / W1-b / W2-a·b·c·d / W6 / W6-b</t>
         </is>
       </c>
       <c r="D4" s="4" t="inlineStr">
@@ -641,11 +641,11 @@
       </c>
       <c r="H4" s="5" t="inlineStr">
         <is>
-          <t>单台 / 多台都做：多台由 ca-api 单机循环调用，不动 micro、不新增批量接口；售货机走单机货道维度。适用机型与建模校验复用后端，AI 只透传失败原因。⚠ 2026-10-16 裁决：① 离线机器同样支持上架，前端不设在线门槛，能否真正下发由后端判定、失败原因透传；② 多机型批量上架时，私有商品库按「本批机器机型的交集」出商品（单台＝该机机型）</t>
-        </is>
-      </c>
-    </row>
-    <row r="5" ht="34" customHeight="1">
+          <t>单台 / 多台都做：多台由 ca-api 单机循环调用，不动 micro、不新增批量接口；售货机走单机货道维度。适用机型与建模校验复用后端，AI 只透传失败原因。⚠ 2026-10-16 裁决：① 离线机器同样支持上架，前端不设在线门槛，能否真正下发由后端判定、失败原因透传；② 多机型批量上架时，私有商品库按「本批机器机型的交集」出商品（单台＝该机机型）；③ 2026-10-28 定稿 19：批量上架改「一张卡内三步向导」——选商品 → 选机器 → **逐台按机型定位置 / 价格 / 库存**（智能柜默认第 1 层、售货机默认下一个空闲货道，预填后仍可点选改；旧口径「批量不逐台指定、各机自动分配」作废）；④ 同日新增「按货道上架」：问法点名货道（「所有机器的 A1 货道上架百事可乐」）→ 位置锁定该货道、直接从第 3 步起、机器范围只留售货机，卡内写明「已跳过 N 台非售货机」；⑤ 同日定稿 20：「批量 / 一键 / 全量」视为范围词，说了就进三步向导第 1 步，不再反问「要在哪台机器上架」</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="132" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>B1</t>
@@ -683,7 +683,7 @@
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>查 ① 最近一月补货机器 + ② 各机补货次数；③ 未补货时长按从长到短倒序</t>
+          <t>⚠ 2026-10-28 定稿 18：查的是「该补还没补的机器」，不是补货流水——口径＝近 30 天 ∩ 在线 ∩ 有销量 ∩ 未补货 &gt; 15 天（三者取交集），按未补货时长倒序（≥21 天标红、&gt;15 天标橙）。三个条件做成卡内可点 chip（默认全开），点掉即在卡内重算、不放宽成「一步一步反问」；kv 给「命中 N 台 / 共 M 台 · 排除 K 台」；命中 0 台走空状态卡并列出被哪个条件滤掉。旧口径「补过货的机器 + 补货次数 + 默认勾中 7 天以上」作废</t>
         </is>
       </c>
     </row>
@@ -1340,7 +1340,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E27"/>
+  <dimension ref="A1:E30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2005,55 +2005,136 @@
         </is>
       </c>
     </row>
-    <row r="26" ht="62" customHeight="1">
-      <c r="A26" s="11" t="inlineStr">
+    <row r="26" ht="300" customHeight="1">
+      <c r="A26" s="4" t="inlineStr">
+        <is>
+          <t>24</t>
+        </is>
+      </c>
+      <c r="B26" s="5" t="inlineStr">
+        <is>
+          <t>补货记录「近 30 天」口径与条件可见（R1 / B1 · 定稿 #18）</t>
+        </is>
+      </c>
+      <c r="C26" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-28 产品反馈（原话「补货记录（近 30 天）：逻辑调整，查最近一个月在线、有销量、未补货时间大于15天的；可以改成一步一步询问的方式」）：**这张卡查的是「该补还没补的机器」，不是补货流水**。口径＝**近 30 天 ∩ 在线 ∩ 有销量 ∩ 未补货 &gt; 15 天**（三者取交集），按未补货时长倒序，≥21 天标红、&gt;15 天标橙。（1）**条件写死但不隐藏**——三个条件在卡内做成**可点 chip**（默认全开），点掉一个条件立刻在卡内重算、不算新提问也不发新请求，让客户自己看出「为什么只有这几台」；kv 行同步给「命中 N 台 / 共 M 台 · 排除 K 台」。（2）**不改成「一步一步反问」**——反问会让客户多点两次还看不到全貌，用户原话里「可以改成」是允许而非要求。（3）**命中 0 台走空状态卡**（`.empty-inline`），不说「没数据」，而是列出前 3 台被哪个条件滤掉的（如「格子柜 A 座（离线）」「梅林一村（近一月无销量）」「欢乐颂 5 号机（仅 13 天）」）。⚠ 旧口径「最近一个月**补过货**的机器 + 各机补货次数 + 默认勾中 7 天以上」作废；演示数据 `REPLEN_REC` 同步重排为 4 命中（21/18/17/16 天）+ 3 类未命中（离线 26 天 / 零销量 19 天 / 13 天未超阈值），保证筛选逻辑在卡内可验证</t>
+        </is>
+      </c>
+      <c r="D26" s="5" t="inlineStr">
+        <is>
+          <t>产品反馈 2026-10-28（附原型截图）；需求说明 §6.1 / §12.1 定稿 #18；卡片设计稿 R1；冒烟 MP 184 / PC 179（R1 相关：命中 4 台且全部 &gt;15 天、离线 / 零销量 / 未超阈值 3 台被排除、kv「排除 5 台」、3 chip 默认全开、点掉「在线」后变 5 台）</t>
+        </is>
+      </c>
+      <c r="E26" s="5" t="inlineStr">
+        <is>
+          <t>已落定，无未决风险</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="356" customHeight="1">
+      <c r="A27" s="4" t="inlineStr">
+        <is>
+          <t>25</t>
+        </is>
+      </c>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>批量上架三步向导 + 按货道上架（W2-a·b·c·d / A1 · 定稿 #19）</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-28 产品反馈（原话「批量上架商品改交互，先选择需要上架的商品，然后选择需要上架的机器，然后根据不同的机器型号在选择货道、价格和库存；智能柜的默认第一层，售货机的需要选择具体的货道」+「新的问答操作：加一个直接通过货道上架商品的操作；比如：所有机器的A1货道上架百事可乐」）：（1）**批量上架改成一张卡内三步向导**——顶部步骤条（选商品 → 选机器 → 位置 / 价格 / 库存），当前步高亮、已完成步打勾、可点「上一步」回改；第 1 步只管上什么（价格可改、补货量默认＝箱规 ×1.5），第 2 步管上到哪（全部 / 按线路 / 自选，沿用 `.seg` 与线路真下拉），第 3 步逐台按机型给位置 + 价格 + 库存（每台一个可展开块，首台默认展开）。（2）**位置＝预填默认 + 可改**：智能柜＝第 1 层（一层不限商品数、不构成占用，见定稿 #14）；售货机＝下一个空闲货道（一货道一商品，副行给最大 · 现存）；点位置 chip 呼出选择弹层（定稿 #13 已有），点选即回填。（3）**新增「按货道上架」（W2-d）**：问法点名货道号 → 位置锁定该货道、直接从第 3 步起、机器范围只留售货机、卡内写明「已跳过 N 台非售货机（智能柜按层管理，无货道编号）」；⚠ 该分支在路由里必须排在通用「批量上架」之前，否则问法里的「上架 / 所有机器」会被通用分支先命中、货道号被吞。⚠ 旧口径「批量不逐台指定货道 / 层，各机自动分配」作废；原实现 12 台 × 3 商品＝36 个位置既看不见也改不了</t>
+        </is>
+      </c>
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>产品反馈 2026-10-28（附原型截图）；需求说明 §4.1 / §4.4 / §5.2 / §9.2 / §12.1 定稿 #19；卡片设计稿 W2-a / W2-b / W2-c（三个界面态）；冒烟 MP 184 / PC 179（W2 相关：第 1 步无机器选择区、步骤条 3 段仅 1 段激活、逐步进入第 2 / 3 步、逐台块＝12 台且首台展开、智能柜默认「第 1 层」、售货机默认形如「A1 货道」、点位置 chip 呼出弹层并回填、确认按钮只在第 3 步；W2-d：直接进第 3 步、位置全锁 A1 货道、块数＝售货机台数、跳过智能柜）</t>
+        </is>
+      </c>
+      <c r="E27" s="5" t="inlineStr">
+        <is>
+          <t>已落定，无未决风险</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="272" customHeight="1">
+      <c r="A28" s="4" t="inlineStr">
+        <is>
+          <t>26</t>
+        </is>
+      </c>
+      <c r="B28" s="5" t="inlineStr">
+        <is>
+          <t>「批量上架」触发词补全（A1 / W2 · 定稿 #20）</t>
+        </is>
+      </c>
+      <c r="C28" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-28 产品反馈（原话「没有对应的卡片交互啊」，附真机截图：输入「批量上架百事可乐」→ AI 反问「请问要在哪台机器上架商品？」→ 用户回「500ml」→ 直接落「这个问题我暂时答不上来」）。根因＝路由里判批量范围的正则只认 `所有机器 / 全部机器 / 所有点位 / 全部点位 / 每台 / 各台`，**不认用户最常用的「批量」二字**——整句带着「批量」却落到最后一行 `askMachine` 去做**单台**补槽位；用户再答商品规格（「500ml」）既不是机器名也没有动作词，被判成「没认出机器」，补槽位超过 2 轮 → 未命中兜底，**一张卡都出不来**。落定：**「批量 / 一键 / 全量」本身就是范围词**，与「所有机器 / 全部点位 / 每台 / 各台」同等处理，命中即进 W2 三步向导第 1 步（选商品），机器范围留到第 2 步再选；只有整句**既无范围词、也未点名机器**（如「上架百事可乐」）才允许反问机器。⚠ 这条是「卡片本身没问题、路由没把用户送进来」的典型：卡片重写时冒烟只钉了「所有机器都上架…」这种标准句式，没覆盖省略范围的裸问法，所以回归全绿也没抓到这个缺陷——已补 MP +2 / PC +1 裸问法断言</t>
+        </is>
+      </c>
+      <c r="D28" s="5" t="inlineStr">
+        <is>
+          <t>产品反馈 2026-10-28（附真机截图）；需求说明 §4.1 / §5.2 / §12.1 定稿 #20；冒烟 MP 184 / PC 179（「批量上架百事可乐」直接出批量向导第 1 步、且不出现「请问要在哪台机器上架商品」）</t>
+        </is>
+      </c>
+      <c r="E28" s="5" t="inlineStr">
+        <is>
+          <t>已落定，无未决风险</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="62" customHeight="1">
+      <c r="A29" s="11" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
-      <c r="B26" s="12" t="inlineStr">
+      <c r="B29" s="12" t="inlineStr">
         <is>
           <t>ca-api 不在代码库（盲区）</t>
         </is>
       </c>
-      <c r="C26" s="5" t="inlineStr">
+      <c r="C29" s="5" t="inlineStr">
         <is>
           <t>B7（NLU 泛化 + 机器点名 / 上下文）与 mp_kb 知识库结构无法在代码层面核对，只能核对到数据源与前端卡片缺口；需 ca-api 侧另行确认</t>
         </is>
       </c>
-      <c r="D26" s="5" t="inlineStr">
+      <c r="D29" s="5" t="inlineStr">
         <is>
           <t>AiChat/api.js:9-13（chat/v2 SSE 与 ca-api 交互）；cardRegistry.js:12-23（现有 10 个能力卡片）</t>
         </is>
       </c>
-      <c r="E26" s="12" t="inlineStr">
+      <c r="E29" s="12" t="inlineStr">
         <is>
           <t>① 接口契约（请求 / 响应 / 错误码）随需求一并冻结，作为联调交付物；② 联调前先用 mock 契约跑通前端卡片；③ 核对不到的部分登记进 §12.2 待确认，不写进卡片文案｜影响：B7 配套能力与 mp_kb 结构无法在代码层核实</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="62" customHeight="1">
-      <c r="A27" s="11" t="inlineStr">
+    <row r="30" ht="62" customHeight="1">
+      <c r="A30" s="11" t="inlineStr">
         <is>
           <t>R2</t>
         </is>
       </c>
-      <c r="B27" s="12" t="inlineStr">
+      <c r="B30" s="12" t="inlineStr">
         <is>
           <t>多台循环上架的部分失败反馈</t>
         </is>
       </c>
-      <c r="C27" s="5" t="inlineStr">
+      <c r="C30" s="5" t="inlineStr">
         <is>
           <t>单机循环时若部分机器被后台校验拦截（不支持机型 / 未绑定商品 code），需逐台列出失败机器与原因，不得整批报失败</t>
         </is>
       </c>
-      <c r="D27" s="5" t="inlineStr">
+      <c r="D30" s="5" t="inlineStr">
         <is>
           <t>与落定口径 1、2 配套，属前端卡片与 ca-api 交互约定</t>
         </is>
       </c>
-      <c r="E27" s="12" t="inlineStr">
+      <c r="E30" s="12" t="inlineStr">
         <is>
           <t>① 结果卡数据模型固定为 {succ[], fail[{机器, 原因}]}，成功 + 失败 = 命中总数；② 后端按机器维度返回错误码，前端原样透传、不改写；③ 重试只对 fail 项重新签发 confirm_id｜影响：批量上下架的结果展示与重试</t>
         </is>

</xml_diff>

<commit_message>
Publish index.html @ 2026-10-28 17:48:45
</commit_message>
<xml_diff>
--- a/iter.xlsx
+++ b/iter.xlsx
@@ -2023,7 +2023,7 @@
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>产品反馈 2026-10-28（附原型截图）；需求说明 §6.1 / §12.1 定稿 #18；卡片设计稿 R1；冒烟 MP 184 / PC 179（R1 相关：命中 4 台且全部 &gt;15 天、离线 / 零销量 / 未超阈值 3 台被排除、kv「排除 5 台」、3 chip 默认全开、点掉「在线」后变 5 台）</t>
+          <t>产品反馈 2026-10-28（附原型截图）；需求说明 §6.1 / §12.1 定稿 #18；卡片设计稿 R1；冒烟 MP 185 / PC 180（R1 相关：命中 4 台且全部 &gt;15 天、离线 / 零销量 / 未超阈值 3 台被排除、kv「排除 5 台」、3 chip 默认全开、点掉「在线」后变 5 台）</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
@@ -2050,7 +2050,7 @@
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>产品反馈 2026-10-28（附原型截图）；需求说明 §4.1 / §4.4 / §5.2 / §9.2 / §12.1 定稿 #19；卡片设计稿 W2-a / W2-b / W2-c（三个界面态）；冒烟 MP 184 / PC 179（W2 相关：第 1 步无机器选择区、步骤条 3 段仅 1 段激活、逐步进入第 2 / 3 步、逐台块＝12 台且首台展开、智能柜默认「第 1 层」、售货机默认形如「A1 货道」、点位置 chip 呼出弹层并回填、确认按钮只在第 3 步；W2-d：直接进第 3 步、位置全锁 A1 货道、块数＝售货机台数、跳过智能柜）</t>
+          <t>产品反馈 2026-10-28（附原型截图）；需求说明 §4.1 / §4.4 / §5.2 / §9.2 / §12.1 定稿 #19；卡片设计稿 W2-a / W2-b / W2-c（三个界面态）；冒烟 MP 185 / PC 180（W2 相关：第 1 步无机器选择区、步骤条 3 段仅 1 段激活、逐步进入第 2 / 3 步、逐台块＝12 台且首台展开、智能柜默认「第 1 层」、售货机默认形如「A1 货道」、点位置 chip 呼出弹层并回填、确认按钮只在第 3 步；W2-d：直接进第 3 步、位置全锁 A1 货道、块数＝售货机台数、跳过智能柜）</t>
         </is>
       </c>
       <c r="E27" s="5" t="inlineStr">
@@ -2059,7 +2059,7 @@
         </is>
       </c>
     </row>
-    <row r="28" ht="272" customHeight="1">
+    <row r="28" ht="342" customHeight="1">
       <c r="A28" s="4" t="inlineStr">
         <is>
           <t>26</t>
@@ -2072,12 +2072,12 @@
       </c>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>2026-10-28 产品反馈（原话「没有对应的卡片交互啊」，附真机截图：输入「批量上架百事可乐」→ AI 反问「请问要在哪台机器上架商品？」→ 用户回「500ml」→ 直接落「这个问题我暂时答不上来」）。根因＝路由里判批量范围的正则只认 `所有机器 / 全部机器 / 所有点位 / 全部点位 / 每台 / 各台`，**不认用户最常用的「批量」二字**——整句带着「批量」却落到最后一行 `askMachine` 去做**单台**补槽位；用户再答商品规格（「500ml」）既不是机器名也没有动作词，被判成「没认出机器」，补槽位超过 2 轮 → 未命中兜底，**一张卡都出不来**。落定：**「批量 / 一键 / 全量」本身就是范围词**，与「所有机器 / 全部点位 / 每台 / 各台」同等处理，命中即进 W2 三步向导第 1 步（选商品），机器范围留到第 2 步再选；只有整句**既无范围词、也未点名机器**（如「上架百事可乐」）才允许反问机器。⚠ 这条是「卡片本身没问题、路由没把用户送进来」的典型：卡片重写时冒烟只钉了「所有机器都上架…」这种标准句式，没覆盖省略范围的裸问法，所以回归全绿也没抓到这个缺陷——已补 MP +2 / PC +1 裸问法断言</t>
+          <t>2026-10-28 产品反馈（原话「没有对应的卡片交互啊」，附真机截图：输入「批量上架百事可乐」→ AI 反问「请问要在哪台机器上架商品？」→ 用户回「500ml」→ 直接落「这个问题我暂时答不上来」）。根因＝路由里判批量范围的正则只认 `所有机器 / 全部机器 / 所有点位 / 全部点位 / 每台 / 各台`，**不认用户最常用的「批量」二字**——整句带着「批量」却落到最后一行 `askMachine` 去做**单台**补槽位；用户再答商品规格（「500ml」）既不是机器名也没有动作词，被判成「没认出机器」，补槽位超过 2 轮 → 未命中兜底，**一张卡都出不来**。落定：**「批量 / 一键 / 全量」本身就是范围词**，与「所有机器 / 全部点位 / 每台 / 各台」同等处理，命中即进 W2 三步向导第 1 步（选商品），机器范围留到第 2 步再选；只有整句**既无范围词、也未点名机器**（如「上架百事可乐」）才允许反问机器。连带修一处：反问分支原写成 `return askMachine(...)`，该函数无返回值、被上层当成「没命中」继续往下走，反问句后面又跟一条「抱歉，我暂时无法回答这个问题」——改为反问后显式结束链路，反问只出一句。⚠ 这条是「卡片本身没问题、路由没把用户送进来」的典型：卡片重写时冒烟只钉了「所有机器都上架…」这种标准句式，没覆盖省略范围的裸问法，所以回归全绿也没抓到这个缺陷——已补 MP +3 / PC +2 裸问法断言（含「上架百事可乐」只反问机器一句、不跟兜底）</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>产品反馈 2026-10-28（附真机截图）；需求说明 §4.1 / §5.2 / §12.1 定稿 #20；冒烟 MP 184 / PC 179（「批量上架百事可乐」直接出批量向导第 1 步、且不出现「请问要在哪台机器上架商品」）</t>
+          <t>产品反馈 2026-10-28（附真机截图）；需求说明 §4.1 / §5.2 / §12.1 定稿 #20；冒烟 MP 185 / PC 180（「批量上架百事可乐」直接出批量向导第 1 步、且不出现「请问要在哪台机器上架商品」）</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">

</xml_diff>

<commit_message>
Publish index.html @ 2026-10-28 18:13:07
</commit_message>
<xml_diff>
--- a/iter.xlsx
+++ b/iter.xlsx
@@ -603,7 +603,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="244" customHeight="1">
+    <row r="4" ht="314" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
           <t>A1</t>
@@ -641,7 +641,7 @@
       </c>
       <c r="H4" s="5" t="inlineStr">
         <is>
-          <t>单台 / 多台都做：多台由 ca-api 单机循环调用，不动 micro、不新增批量接口；售货机走单机货道维度。适用机型与建模校验复用后端，AI 只透传失败原因。⚠ 2026-10-16 裁决：① 离线机器同样支持上架，前端不设在线门槛，能否真正下发由后端判定、失败原因透传；② 多机型批量上架时，私有商品库按「本批机器机型的交集」出商品（单台＝该机机型）；③ 2026-10-28 定稿 19：批量上架改「一张卡内三步向导」——选商品 → 选机器 → **逐台按机型定位置 / 价格 / 库存**（智能柜默认第 1 层、售货机默认下一个空闲货道，预填后仍可点选改；旧口径「批量不逐台指定、各机自动分配」作废）；④ 同日新增「按货道上架」：问法点名货道（「所有机器的 A1 货道上架百事可乐」）→ 位置锁定该货道、直接从第 3 步起、机器范围只留售货机，卡内写明「已跳过 N 台非售货机」；⑤ 同日定稿 20：「批量 / 一键 / 全量」视为范围词，说了就进三步向导第 1 步，不再反问「要在哪台机器上架」</t>
+          <t>单台 / 多台都做：多台由 ca-api 单机循环调用，不动 micro、不新增批量接口；售货机走单机货道维度。适用机型与建模校验复用后端，AI 只透传失败原因。⚠ 2026-10-16 裁决：① 离线机器同样支持上架，前端不设在线门槛，能否真正下发由后端判定、失败原因透传；② 多机型批量上架时，私有商品库按「本批机器机型的交集」出商品（单台＝该机机型）；③ 2026-10-28 定稿 19 / 21：批量上架改「一张卡内三步向导」——选商品 → 选机器 → **按机型统一设置位置 / 价格 / 库存**（同一机型只给一行：智能柜＝层、售货机＝起始货道并逐台按各自空闲货道顺延；预填后仍可点选改；定稿 19 的「逐台一个块」已被 21 取代）；④ 同日新增「按货道上架」：问法点名货道（「所有机器的 A1 货道上架百事可乐」）→ 位置锁定该货道、直接从第 3 步起、机器范围只留售货机，卡内写明「已跳过 N 台非售货机」；⑤ 同日定稿 20：「批量 / 一键 / 全量」视为范围词，说了就进三步向导第 1 步，不再反问「要在哪台机器上架」；⑥ 同日定稿 22：第 2 步撤下「全部机器」档，只留「按线路 / 自选」（范围词仍进卡，进卡后默认第一条线路）；⑦ 同日定稿 23：第 1 步商品行可「✕ 移除」、可删到 0 并给空态 + 禁用下一步</t>
         </is>
       </c>
     </row>
@@ -1340,7 +1340,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E30"/>
+  <dimension ref="A1:E33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2023,7 +2023,7 @@
       </c>
       <c r="D26" s="5" t="inlineStr">
         <is>
-          <t>产品反馈 2026-10-28（附原型截图）；需求说明 §6.1 / §12.1 定稿 #18；卡片设计稿 R1；冒烟 MP 185 / PC 180（R1 相关：命中 4 台且全部 &gt;15 天、离线 / 零销量 / 未超阈值 3 台被排除、kv「排除 5 台」、3 chip 默认全开、点掉「在线」后变 5 台）</t>
+          <t>产品反馈 2026-10-28（附原型截图）；需求说明 §6.1 / §12.1 定稿 #18；卡片设计稿 R1；冒烟 MP 191 / PC 184（R1 相关：命中 4 台且全部 &gt;15 天、离线 / 零销量 / 未超阈值 3 台被排除、kv「排除 5 台」、3 chip 默认全开、点掉「在线」后变 5 台）</t>
         </is>
       </c>
       <c r="E26" s="5" t="inlineStr">
@@ -2050,7 +2050,7 @@
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>产品反馈 2026-10-28（附原型截图）；需求说明 §4.1 / §4.4 / §5.2 / §9.2 / §12.1 定稿 #19；卡片设计稿 W2-a / W2-b / W2-c（三个界面态）；冒烟 MP 185 / PC 180（W2 相关：第 1 步无机器选择区、步骤条 3 段仅 1 段激活、逐步进入第 2 / 3 步、逐台块＝12 台且首台展开、智能柜默认「第 1 层」、售货机默认形如「A1 货道」、点位置 chip 呼出弹层并回填、确认按钮只在第 3 步；W2-d：直接进第 3 步、位置全锁 A1 货道、块数＝售货机台数、跳过智能柜）</t>
+          <t>产品反馈 2026-10-28（附原型截图）；需求说明 §4.1 / §4.4 / §5.2 / §9.2 / §12.1 定稿 #19；卡片设计稿 W2-a / W2-b / W2-c（三个界面态）；冒烟 MP 191 / PC 184（W2 相关：第 1 步无机器选择区、步骤条 3 段仅 1 段激活、逐步进入第 2 / 3 步、第 3 步按机型分组（3 台两机型只出 2 块、块头「N 台 · 统一设置」、行数＝机型数 × 商品数）、智能柜默认「第 1 层」、售货机默认形如「A1 货道」、点位置 chip 呼出弹层并回填、确认按钮只在第 3 步；W2-d：直接进第 3 步、位置全锁 A1 货道、多台售货机合成 1 块、跳过智能柜）</t>
         </is>
       </c>
       <c r="E27" s="5" t="inlineStr">
@@ -2077,7 +2077,7 @@
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>产品反馈 2026-10-28（附真机截图）；需求说明 §4.1 / §5.2 / §12.1 定稿 #20；冒烟 MP 185 / PC 180（「批量上架百事可乐」直接出批量向导第 1 步、且不出现「请问要在哪台机器上架商品」）</t>
+          <t>产品反馈 2026-10-28（附真机截图）；需求说明 §4.1 / §5.2 / §12.1 定稿 #20；冒烟 MP 191 / PC 184（「批量上架百事可乐」直接出批量向导第 1 步、且不出现「请问要在哪台机器上架商品」）</t>
         </is>
       </c>
       <c r="E28" s="5" t="inlineStr">
@@ -2086,55 +2086,136 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="62" customHeight="1">
-      <c r="A29" s="11" t="inlineStr">
+    <row r="29" ht="258" customHeight="1">
+      <c r="A29" s="4" t="inlineStr">
+        <is>
+          <t>27</t>
+        </is>
+      </c>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>批量上架第 3 步改按机型统一设置（W2-a / A1 · 定稿 #21）</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-28 产品反馈（原话「我要的其实是智能柜都选一个层数价格和库存上架，售货机同理，而不是到这一步后还是要一台台机器的设置库存价格等」）：第 3 步**不再逐台一个块**。① **同一机型只给一行**——智能柜 N 台＝一行「层 + 价格 + 库存」，售货机 M 台＝一行「起始货道 + 价格 + 库存」；块头写「售货机 / 智能柜 · N 台 · 统一设置」，表头「商品 / 起始货道（或层）/ 价格 / 库存」。② **售货机货道顺延**：一行只填起始货道，提交时每台机器**从该起始货道起、按自己未占用的货道依次顺延**（`lanesFrom(m,start,n)`；已占用货道自动跳过）；点名具体货道（W2-d）不加顺延、全部锁死该货道。③ 预览写「售货机 N 台 · 从「A1 货道」起 · 每台按各自空闲货道顺延」/「智能柜 N 台 · 统一放「第 1 层」」；确认按钮 N＝总台数不＝行数。⚠ 原方案 12 台 × 3 商品＝36 个位置要一台台设置，而同一批机器上同一批商品价格库存本来就一样，逐台没有信息量；定稿 #19 的「逐台一个块、首台展开」被本条取代</t>
+        </is>
+      </c>
+      <c r="D29" s="5" t="inlineStr">
+        <is>
+          <t>产品反馈 2026-10-28（附真机截图）；需求说明 §5.2 / §9.2 / §12.1 定稿 #21；卡片设计稿 W2-a / W2-b / W2-c；冒烟 MP 191 / PC 184（3 台两机型只出 2 块、块头「N 台 · 统一设置」、行数＝机型数 × 商品数、智能柜默认第 1 层、售货机起始货道形如「A1 货道」）</t>
+        </is>
+      </c>
+      <c r="E29" s="5" t="inlineStr">
+        <is>
+          <t>已落定，无未决风险</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="160" customHeight="1">
+      <c r="A30" s="4" t="inlineStr">
+        <is>
+          <t>28</t>
+        </is>
+      </c>
+      <c r="B30" s="5" t="inlineStr">
+        <is>
+          <t>批量上架撤下「全部机器」档（W2-a / A1 · 定稿 #22）</t>
+        </is>
+      </c>
+      <c r="C30" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-28 产品反馈（原话「不要全部机器了，让客户按线路或者自选」）：第 2 步 `.seg` 只留**「按线路 / 自选」两档**，默认按线路。⚠ **范围词与档位解耦**——「所有机器 / 全部机器 / 批量 / 一键 / 全量」这类问法**仍然进卡**（不能因为档位撤了就反问机器），但进卡后范围**默认落第一条线路**，客户自己改线路或切「自选」。理由：批量上架是写操作，影响面必须收窄到客户能核对的范围。⚠ 连带调整：W6 结果卡原来靠「全部 12 台」制造 10 成功 / 2 失败的混合结果，档位撤下后改用「科技园线路」（3 台，含不支持上架的格子柜）复现 2 成功 / 1 失败，两端冒烟同步改问法与断言</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>产品反馈 2026-10-28（附真机截图）；需求说明 §4.1 / §4.4 / §5.2 / §12.1 定稿 #22；卡片设计稿 W2-b；冒烟 MP 191 / PC 184（`.seg` 只剩 2 档、卡内不出现「全部机器」）</t>
+        </is>
+      </c>
+      <c r="E30" s="5" t="inlineStr">
+        <is>
+          <t>已落定，无未决风险</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="104" customHeight="1">
+      <c r="A31" s="4" t="inlineStr">
+        <is>
+          <t>29</t>
+        </is>
+      </c>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>第 1 步商品可删除（W2-a / P1 · 定稿 #23）</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-28 产品反馈（原话「我才发现只有添加没有删除商品的操作」）：每个商品行右侧补「✕ 移除」，点了即从本卡移除（含刚在 P1 弹层里加的）；**允许删到 0**——删空后第 1 步给空态「还没有商品 —— 点下面「＋ 添加商品」挑一个」，底部「下一步」置灰并提示「请至少保留一个商品」。原实现只在「添加」方向有入口，选错商品只能关掉整张卡重开</t>
+        </is>
+      </c>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>产品反馈 2026-10-28（附真机截图）；需求说明 §5.2 / §12.1 定稿 #23；卡片设计稿 W2-a；冒烟 MP 191 / PC 184（`.pdel` 数＝商品行数、点 ✕ 后行数 −1、删空出现「还没有商品」且 `_next` 置灰）</t>
+        </is>
+      </c>
+      <c r="E31" s="5" t="inlineStr">
+        <is>
+          <t>已落定，无未决风险</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="62" customHeight="1">
+      <c r="A32" s="11" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
-      <c r="B29" s="12" t="inlineStr">
+      <c r="B32" s="12" t="inlineStr">
         <is>
           <t>ca-api 不在代码库（盲区）</t>
         </is>
       </c>
-      <c r="C29" s="5" t="inlineStr">
+      <c r="C32" s="5" t="inlineStr">
         <is>
           <t>B7（NLU 泛化 + 机器点名 / 上下文）与 mp_kb 知识库结构无法在代码层面核对，只能核对到数据源与前端卡片缺口；需 ca-api 侧另行确认</t>
         </is>
       </c>
-      <c r="D29" s="5" t="inlineStr">
+      <c r="D32" s="5" t="inlineStr">
         <is>
           <t>AiChat/api.js:9-13（chat/v2 SSE 与 ca-api 交互）；cardRegistry.js:12-23（现有 10 个能力卡片）</t>
         </is>
       </c>
-      <c r="E29" s="12" t="inlineStr">
+      <c r="E32" s="12" t="inlineStr">
         <is>
           <t>① 接口契约（请求 / 响应 / 错误码）随需求一并冻结，作为联调交付物；② 联调前先用 mock 契约跑通前端卡片；③ 核对不到的部分登记进 §12.2 待确认，不写进卡片文案｜影响：B7 配套能力与 mp_kb 结构无法在代码层核实</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="62" customHeight="1">
-      <c r="A30" s="11" t="inlineStr">
+    <row r="33" ht="62" customHeight="1">
+      <c r="A33" s="11" t="inlineStr">
         <is>
           <t>R2</t>
         </is>
       </c>
-      <c r="B30" s="12" t="inlineStr">
+      <c r="B33" s="12" t="inlineStr">
         <is>
           <t>多台循环上架的部分失败反馈</t>
         </is>
       </c>
-      <c r="C30" s="5" t="inlineStr">
+      <c r="C33" s="5" t="inlineStr">
         <is>
           <t>单机循环时若部分机器被后台校验拦截（不支持机型 / 未绑定商品 code），需逐台列出失败机器与原因，不得整批报失败</t>
         </is>
       </c>
-      <c r="D30" s="5" t="inlineStr">
+      <c r="D33" s="5" t="inlineStr">
         <is>
           <t>与落定口径 1、2 配套，属前端卡片与 ca-api 交互约定</t>
         </is>
       </c>
-      <c r="E30" s="12" t="inlineStr">
+      <c r="E33" s="12" t="inlineStr">
         <is>
           <t>① 结果卡数据模型固定为 {succ[], fail[{机器, 原因}]}，成功 + 失败 = 命中总数；② 后端按机器维度返回错误码，前端原样透传、不改写；③ 重试只对 fail 项重新签发 confirm_id｜影响：批量上下架的结果展示与重试</t>
         </is>

</xml_diff>

<commit_message>
Publish index.html @ 2026-10-28 19:02:22
</commit_message>
<xml_diff>
--- a/iter.xlsx
+++ b/iter.xlsx
@@ -603,7 +603,7 @@
         </is>
       </c>
     </row>
-    <row r="4" ht="314" customHeight="1">
+    <row r="4" ht="440" customHeight="1">
       <c r="A4" s="4" t="inlineStr">
         <is>
           <t>A1</t>
@@ -641,7 +641,7 @@
       </c>
       <c r="H4" s="5" t="inlineStr">
         <is>
-          <t>单台 / 多台都做：多台由 ca-api 单机循环调用，不动 micro、不新增批量接口；售货机走单机货道维度。适用机型与建模校验复用后端，AI 只透传失败原因。⚠ 2026-10-16 裁决：① 离线机器同样支持上架，前端不设在线门槛，能否真正下发由后端判定、失败原因透传；② 多机型批量上架时，私有商品库按「本批机器机型的交集」出商品（单台＝该机机型）；③ 2026-10-28 定稿 19 / 21：批量上架改「一张卡内三步向导」——选商品 → 选机器 → **按机型统一设置位置 / 价格 / 库存**（同一机型只给一行：智能柜＝层、售货机＝起始货道并逐台按各自空闲货道顺延；预填后仍可点选改；定稿 19 的「逐台一个块」已被 21 取代）；④ 同日新增「按货道上架」：问法点名货道（「所有机器的 A1 货道上架百事可乐」）→ 位置锁定该货道、直接从第 3 步起、机器范围只留售货机，卡内写明「已跳过 N 台非售货机」；⑤ 同日定稿 20：「批量 / 一键 / 全量」视为范围词，说了就进三步向导第 1 步，不再反问「要在哪台机器上架」；⑥ 同日定稿 22：第 2 步撤下「全部机器」档，只留「按线路 / 自选」（范围词仍进卡，进卡后默认第一条线路）；⑦ 同日定稿 23：第 1 步商品行可「✕ 移除」、可删到 0 并给空态 + 禁用下一步</t>
+          <t>单台 / 多台都做：多台由 ca-api 单机循环调用，不动 micro、不新增批量接口；售货机走单机货道维度。适用机型与建模校验复用后端，AI 只透传失败原因。⚠ 2026-10-16 裁决：① 离线机器同样支持上架，前端不设在线门槛，能否真正下发由后端判定、失败原因透传；② 多机型批量上架时，私有商品库按「本批机器机型的交集」出商品（单台＝该机机型）；③ 2026-10-28 定稿 19 / 21：批量上架改「一张卡内三步向导」——选商品 → 选机器 → **按机型统一设置位置 / 价格 / 库存**（同一机型只给一行：智能柜＝层、售货机＝起始货道并逐台按各自空闲货道顺延；预填后仍可点选改；定稿 19 的「逐台一个块」已被 21 取代）；④ 同日新增「按货道上架」：问法点名货道（「所有机器的 A1 货道上架百事可乐」）→ 位置锁定该货道、直接从第 3 步起、机器范围只留售货机，卡内写明「已跳过 N 台非售货机」；⑤ 同日定稿 20：「批量 / 一键 / 全量」视为范围词，说了就进三步向导第 1 步，不再反问「要在哪台机器上架」；⑥ 同日定稿 22：第 2 步撤下「全部机器」档，只留「按线路 / 自选」（范围词仍进卡，进卡后默认第一条线路）；⑦ 同日定稿 23：第 1 步商品行可「✕ 移除」、可删到 0 并给空态 + 禁用下一步；⑧ 同日定稿 24：售货机**一货道一商品**——同卡内两个商品不能选同一货道（默认各占不同空闲货道；选择弹层里被本卡占的货道置灰标「本卡已占用」、点了只提示不改选；提交按每个商品各自的货道落位、该机被占时顺延，货道号先归一化再比）；⑨ 同日定稿 25：**不可上架的机器在选机器阶段就剔除**（机型不支持 / 商品未建模），不进第 3 步、不计入确认台数，卡内写「已跳过 N 台不可上架的机器：名称（原因）」；单台点名到这类机器走「这台机器上架不了」说明卡，不出写卡</t>
         </is>
       </c>
     </row>
@@ -1340,7 +1340,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E33"/>
+  <dimension ref="A1:E35"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2086,7 +2086,7 @@
         </is>
       </c>
     </row>
-    <row r="29" ht="258" customHeight="1">
+    <row r="29" ht="314" customHeight="1">
       <c r="A29" s="4" t="inlineStr">
         <is>
           <t>27</t>
@@ -2099,7 +2099,7 @@
       </c>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>2026-10-28 产品反馈（原话「我要的其实是智能柜都选一个层数价格和库存上架，售货机同理，而不是到这一步后还是要一台台机器的设置库存价格等」）：第 3 步**不再逐台一个块**。① **同一机型只给一行**——智能柜 N 台＝一行「层 + 价格 + 库存」，售货机 M 台＝一行「起始货道 + 价格 + 库存」；块头写「售货机 / 智能柜 · N 台 · 统一设置」，表头「商品 / 起始货道（或层）/ 价格 / 库存」。② **售货机货道顺延**：一行只填起始货道，提交时每台机器**从该起始货道起、按自己未占用的货道依次顺延**（`lanesFrom(m,start,n)`；已占用货道自动跳过）；点名具体货道（W2-d）不加顺延、全部锁死该货道。③ 预览写「售货机 N 台 · 从「A1 货道」起 · 每台按各自空闲货道顺延」/「智能柜 N 台 · 统一放「第 1 层」」；确认按钮 N＝总台数不＝行数。⚠ 原方案 12 台 × 3 商品＝36 个位置要一台台设置，而同一批机器上同一批商品价格库存本来就一样，逐台没有信息量；定稿 #19 的「逐台一个块、首台展开」被本条取代</t>
+          <t>2026-10-28 产品反馈（原话「我要的其实是智能柜都选一个层数价格和库存上架，售货机同理，而不是到这一步后还是要一台台机器的设置库存价格等」）：第 3 步**不再逐台一个块**。① **同一机型只给一行**——智能柜 N 台＝一行「层 + 价格 + 库存」，售货机 M 台＝一行「起始货道 + 价格 + 库存」；块头写「售货机 / 智能柜 · N 台 · 统一设置」，表头「商品 / 起始货道（或层）/ 价格 / 库存」。② **售货机货道顺延**：一行只填起始货道，提交时每台机器**从该起始货道起、按自己未占用的货道依次顺延**（`lanesFrom(m,start,n)`；已占用货道自动跳过）；点名具体货道（W2-d）不加顺延、全部锁死该货道。③ 预览写「售货机 N 台 · 从「A1 货道」起 · 每台按各自空闲货道顺延」/「智能柜 N 台 · 统一放「第 1 层」」；确认按钮 N＝总台数不＝行数。⚠ 原方案 12 台 × 3 商品＝36 个位置要一台台设置，而同一批机器上同一批商品价格库存本来就一样，逐台没有信息量；定稿 #19 的「逐台一个块、首台展开」被本条取代。⚠ **位置口径已被 #24 收敛**：售货机从「一行只填起始货道、逐台顺延」改为**每个商品各自的货道**（默认互不相同，提交按各自货道落位、被占才顺延），预览文案同步改「售货机 N 台 · A2 / A4 · 每台按各自空闲货道落位」</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
@@ -2113,7 +2113,7 @@
         </is>
       </c>
     </row>
-    <row r="30" ht="160" customHeight="1">
+    <row r="30" ht="230" customHeight="1">
       <c r="A30" s="4" t="inlineStr">
         <is>
           <t>28</t>
@@ -2126,7 +2126,7 @@
       </c>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>2026-10-28 产品反馈（原话「不要全部机器了，让客户按线路或者自选」）：第 2 步 `.seg` 只留**「按线路 / 自选」两档**，默认按线路。⚠ **范围词与档位解耦**——「所有机器 / 全部机器 / 批量 / 一键 / 全量」这类问法**仍然进卡**（不能因为档位撤了就反问机器），但进卡后范围**默认落第一条线路**，客户自己改线路或切「自选」。理由：批量上架是写操作，影响面必须收窄到客户能核对的范围。⚠ 连带调整：W6 结果卡原来靠「全部 12 台」制造 10 成功 / 2 失败的混合结果，档位撤下后改用「科技园线路」（3 台，含不支持上架的格子柜）复现 2 成功 / 1 失败，两端冒烟同步改问法与断言</t>
+          <t>2026-10-28 产品反馈（原话「不要全部机器了，让客户按线路或者自选」）：第 2 步 `.seg` 只留**「按线路 / 自选」两档**，默认按线路。⚠ **范围词与档位解耦**——「所有机器 / 全部机器 / 批量 / 一键 / 全量」这类问法**仍然进卡**（不能因为档位撤了就反问机器），但进卡后范围**默认落第一条线路**，客户自己改线路或切「自选」。理由：批量上架是写操作，影响面必须收窄到客户能核对的范围。⚠ 连带调整：W6 结果卡原来靠「全部 12 台」制造 10 成功 / 2 失败的混合结果，档位撤下后改用「科技园线路」（3 台，含不支持上架的格子柜）复现 2 成功 / 1 失败，两端冒烟同步改问法与断言。⚠ **该复现路径已被 #25 取代**：不可上架的格子柜在「选机器」阶段就被剔除，科技园线路只剩 2 台全成功——W6 部分失败改由**运行期兜底**（并发改价 / 机器离线 / 权限变更）触发，冒烟直接用 `cardBatchResult` 出卡验 UI，不再伪装成一次用户旅程</t>
         </is>
       </c>
       <c r="D30" s="5" t="inlineStr">
@@ -2167,55 +2167,109 @@
         </is>
       </c>
     </row>
-    <row r="32" ht="62" customHeight="1">
-      <c r="A32" s="11" t="inlineStr">
+    <row r="32" ht="258" customHeight="1">
+      <c r="A32" s="4" t="inlineStr">
+        <is>
+          <t>30</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr">
+        <is>
+          <t>售货机货道互斥（W2-a / W1 · 定稿 #24）</t>
+        </is>
+      </c>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-28 产品反馈（原话「批量上架商品售货机选择货道这里要做个限制，比如商品a选了A1货道，商品b就不能在选择这个货道了，不然会有问题无法上架商品」，附真机截图：两个商品都选了 A1 货道）：售货机是「一货道一商品」，提交时后写的覆盖先写的、后端只成功一条，客户看到的是「操作成功、其实只上架了一个商品」。① **默认就分开**：第 3 步售货机块里每个商品行各有一个货道 chip，默认按商品顺序取**不同的空闲货道**（不再两个商品都给 A1）。② **弹层互斥**：本卡其它商品已占的货道置灰、写「本卡已占用：X · 选别的货道」，点了只弹提示、不改选择，其余货道照常可选。③ **提交按每个商品各自的货道落位**，该机上那个货道被别人占着就顺延到最近的空闲货道（同卡内已分配的也算占用）；⚠ 点名货道（W2-d）不加顺延、全部锁死。④ 根因补充：演示数据里货道号写法不统一（`A3` / `A1 货道` / `1号货道`），原来按字符串直比会把机器上**已有的 A1 当成空闲**、默认位置就撞道——占用判断统一先归一化再比（`laneKey`）</t>
+        </is>
+      </c>
+      <c r="D32" s="5" t="inlineStr">
+        <is>
+          <t>产品反馈 2026-10-28（附真机截图）；需求说明 §5.2 / §12.1 定稿 #24；卡片设计稿 W2-c；冒烟 MP 200 / PC 187（W2-h：同卡两商品默认不同货道、弹层置灰行标「本卡已占用」、点置灰行不改选择、空闲货道可正常切换）</t>
+        </is>
+      </c>
+      <c r="E32" s="5" t="inlineStr">
+        <is>
+          <t>已落定，无未决风险</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="314" customHeight="1">
+      <c r="A33" s="4" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>不可上架机型前置过滤（W1 / W2-a·b·c · 定稿 #25）</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-28 产品反馈（原话「还有就是直接过滤掉商品不可售的机型，而不是说在提交后才提示用户不可上架」）：原来「机型不支持上架 / 商品未建模」要等客户填完价格库存、点了确认，才在 W6 结果卡里报失败。改为**在选机器阶段就剔除**：① 过滤条件两条——机型本身不支持上架（格子柜）、商品在这台机器上未建模（未绑定可售机型商品 code）；② 命中的机器**不进第 3 步、不计入「确认上架（N 台）」**，卡内在范围下方写「已跳过 N 台不可上架的机器：机器名（原因）」（第 2 步与第 3 步都显示）；③ 改线路 / 切自选 / 加减商品**都会重新过滤**——卡内保留两份数据（客户选的范围 vs 过滤后能上架的机器），否则一过滤就把客户的选择抹掉了；④ **单台点名**到这类机器（「在格子柜 A 座上架百事可乐」）→ 直接给「这台机器上架不了」说明卡（机器 / 机型 / 商品 + 原因 + 下一步 + 未提交任何变更），不摆写卡、不给确认按钮。⚠ 连带修：批量上架**全成功态**原来借单台卡的收尾函数 `finishOp`，它写的是单台卡的 `_op` 包裹层，批量卡没有这层 → 会卡在「⏳ 执行中…」什么也不出（#25 之后批量第一次真的能全成功，才暴露这个缺陷）；改为在本卡内收尾。⚠ W6 结果卡退回**运行期兜底**（并发改价 / 机器离线 / 权限变更）</t>
+        </is>
+      </c>
+      <c r="D33" s="5" t="inlineStr">
+        <is>
+          <t>产品反馈 2026-10-28（附真机截图）；需求说明 §5.1 / §5.2 / §5.6 / §12.1 定稿 #25；卡片设计稿 W2-b；冒烟 MP 200 / PC 187（第 2 步「已跳过 N 台不可上架的机器」含机器名与原因、第 3 步台数不含被剔除机器、批量全成功不产生失败项、单台点名不可上架机型走说明卡且无写卡 / 无确认按钮、格子柜与未建模商品两条路径各一条）</t>
+        </is>
+      </c>
+      <c r="E33" s="5" t="inlineStr">
+        <is>
+          <t>已落定，无未决风险</t>
+        </is>
+      </c>
+    </row>
+    <row r="34" ht="62" customHeight="1">
+      <c r="A34" s="11" t="inlineStr">
         <is>
           <t>R1</t>
         </is>
       </c>
-      <c r="B32" s="12" t="inlineStr">
+      <c r="B34" s="12" t="inlineStr">
         <is>
           <t>ca-api 不在代码库（盲区）</t>
         </is>
       </c>
-      <c r="C32" s="5" t="inlineStr">
+      <c r="C34" s="5" t="inlineStr">
         <is>
           <t>B7（NLU 泛化 + 机器点名 / 上下文）与 mp_kb 知识库结构无法在代码层面核对，只能核对到数据源与前端卡片缺口；需 ca-api 侧另行确认</t>
         </is>
       </c>
-      <c r="D32" s="5" t="inlineStr">
+      <c r="D34" s="5" t="inlineStr">
         <is>
           <t>AiChat/api.js:9-13（chat/v2 SSE 与 ca-api 交互）；cardRegistry.js:12-23（现有 10 个能力卡片）</t>
         </is>
       </c>
-      <c r="E32" s="12" t="inlineStr">
+      <c r="E34" s="12" t="inlineStr">
         <is>
           <t>① 接口契约（请求 / 响应 / 错误码）随需求一并冻结，作为联调交付物；② 联调前先用 mock 契约跑通前端卡片；③ 核对不到的部分登记进 §12.2 待确认，不写进卡片文案｜影响：B7 配套能力与 mp_kb 结构无法在代码层核实</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="62" customHeight="1">
-      <c r="A33" s="11" t="inlineStr">
+    <row r="35" ht="62" customHeight="1">
+      <c r="A35" s="11" t="inlineStr">
         <is>
           <t>R2</t>
         </is>
       </c>
-      <c r="B33" s="12" t="inlineStr">
+      <c r="B35" s="12" t="inlineStr">
         <is>
           <t>多台循环上架的部分失败反馈</t>
         </is>
       </c>
-      <c r="C33" s="5" t="inlineStr">
+      <c r="C35" s="5" t="inlineStr">
         <is>
           <t>单机循环时若部分机器被后台校验拦截（不支持机型 / 未绑定商品 code），需逐台列出失败机器与原因，不得整批报失败</t>
         </is>
       </c>
-      <c r="D33" s="5" t="inlineStr">
+      <c r="D35" s="5" t="inlineStr">
         <is>
           <t>与落定口径 1、2 配套，属前端卡片与 ca-api 交互约定</t>
         </is>
       </c>
-      <c r="E33" s="12" t="inlineStr">
+      <c r="E35" s="12" t="inlineStr">
         <is>
           <t>① 结果卡数据模型固定为 {succ[], fail[{机器, 原因}]}，成功 + 失败 = 命中总数；② 后端按机器维度返回错误码，前端原样透传、不改写；③ 重试只对 fail 项重新签发 confirm_id｜影响：批量上下架的结果展示与重试</t>
         </is>

</xml_diff>

<commit_message>
Publish index.html @ 2026-10-29 09:33:06
</commit_message>
<xml_diff>
--- a/iter.xlsx
+++ b/iter.xlsx
@@ -645,7 +645,7 @@
         </is>
       </c>
     </row>
-    <row r="5" ht="132" customHeight="1">
+    <row r="5" ht="202" customHeight="1">
       <c r="A5" s="4" t="inlineStr">
         <is>
           <t>B1</t>
@@ -683,7 +683,7 @@
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>⚠ 2026-10-28 定稿 18：查的是「该补还没补的机器」，不是补货流水——口径＝近 30 天 ∩ 在线 ∩ 有销量 ∩ 未补货 &gt; 15 天（三者取交集），按未补货时长倒序（≥21 天标红、&gt;15 天标橙）。三个条件做成卡内可点 chip（默认全开），点掉即在卡内重算、不放宽成「一步一步反问」；kv 给「命中 N 台 / 共 M 台 · 排除 K 台」；命中 0 台走空状态卡并列出被哪个条件滤掉。旧口径「补过货的机器 + 补货次数 + 默认勾中 7 天以上」作废</t>
+          <t>⚠ 2026-10-28 定稿 #26：商品级不可售（商品在该机未绑定可售机型商品 code）**不连带整台机器** —— 机器保留在范围内、只跳过这一条组合（第 2 / 3 步提前写明、预览与按钮按条扣减、提交时跳过）；只有**整机级**（机型不支持上架）才在选机器阶段整台剔除。⚠ 2026-10-28 定稿 18：查的是「该补还没补的机器」，不是补货流水——口径＝近 30 天 ∩ 在线 ∩ 有销量 ∩ 未补货 &gt; 15 天（三者取交集），按未补货时长倒序（≥21 天标红、&gt;15 天标橙）。三个条件做成卡内可点 chip（默认全开），点掉即在卡内重算、不放宽成「一步一步反问」；kv 给「命中 N 台 / 共 M 台 · 排除 K 台」；命中 0 台走空状态卡并列出被哪个条件滤掉。旧口径「补过货的机器 + 补货次数 + 默认勾中 7 天以上」作废</t>
         </is>
       </c>
     </row>
@@ -1340,7 +1340,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E35"/>
+  <dimension ref="A1:E36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2202,7 +2202,8 @@
       </c>
       <c r="B33" s="5" t="inlineStr">
         <is>
-          <t>不可上架机型前置过滤（W1 / W2-a·b·c · 定稿 #25）</t>
+          <t>不可上架机型前置过滤（W1 / W2-a·b·c · 定稿 #25）
+⚠ 商品级部分已被落定口径 #32（定稿 #26）回退 —— 现只对**整机级**成立</t>
         </is>
       </c>
       <c r="C33" s="5" t="inlineStr">
@@ -2212,7 +2213,7 @@
       </c>
       <c r="D33" s="5" t="inlineStr">
         <is>
-          <t>产品反馈 2026-10-28（附真机截图）；需求说明 §5.1 / §5.2 / §5.6 / §12.1 定稿 #25；卡片设计稿 W2-b；冒烟 MP 200 / PC 187（第 2 步「已跳过 N 台不可上架的机器」含机器名与原因、第 3 步台数不含被剔除机器、批量全成功不产生失败项、单台点名不可上架机型走说明卡且无写卡 / 无确认按钮、格子柜与未建模商品两条路径各一条）</t>
+          <t>产品反馈 2026-10-28（附真机截图）；需求说明 §5.1 / §5.2 / §5.6 / §12.1 定稿 #25；卡片设计稿 W2-b；冒烟 MP 214 / PC 190（第 2 步「已跳过 N 台不可上架的机器」含机器名与原因、第 3 步台数不含被剔除机器、批量全成功不产生失败项、格子柜整机级走说明卡且无写卡 / 无确认按钮）。⚠ 原「未建模商品也整台剔除」已作废，见落定口径 #32</t>
         </is>
       </c>
       <c r="E33" s="5" t="inlineStr">
@@ -2221,55 +2222,82 @@
         </is>
       </c>
     </row>
-    <row r="34" ht="62" customHeight="1">
-      <c r="A34" s="11" t="inlineStr">
-        <is>
-          <t>R1</t>
-        </is>
-      </c>
-      <c r="B34" s="12" t="inlineStr">
-        <is>
-          <t>ca-api 不在代码库（盲区）</t>
+    <row r="34" ht="482" customHeight="1">
+      <c r="A34" s="4" t="inlineStr">
+        <is>
+          <t>32</t>
+        </is>
+      </c>
+      <c r="B34" s="5" t="inlineStr">
+        <is>
+          <t>商品级不可售要不要连带整台机器（W1 / W2-a·b·c · 定稿 #26 · 回退 #25 的商品级部分）</t>
         </is>
       </c>
       <c r="C34" s="5" t="inlineStr">
         <is>
-          <t>B7（NLU 泛化 + 机器点名 / 上下文）与 mp_kb 知识库结构无法在代码层面核对，只能核对到数据源与前端卡片缺口；需 ca-api 侧另行确认</t>
+          <t>2026-10-28 产品反馈（原话「直接强制不给选机器的话，会出现商品1可以在智能柜上架，但商品2不可以，这样导致智能柜都选不了了」）：定稿 #25 把「机型不支持上架」与「商品在该机未建模」当成同一类，**只要这批商品里有任何一个在这台机器上不了，整台机器就被剔除** —— 但商品级不可售**只影响「这台机器 × 这个商品」这一条组合**，按机器粒度处理会连累能上架的其它商品。⚠⚠ **两级粒度拆开**：① **整机级**（机型不支持上架，如格子柜）＝这台任何商品都上不了 → 保留「选机器阶段整台剔除」；② **商品级**（未绑定可售机型商品 code）＝**机器保留在范围内、只跳过这一条组合**。落地四步：（a）拦截函数拆成 `machineBlockReason(mid)` / `goodsBlockReason(mid,n)` / `blockedPairs(mids,items)`，原 `onshelfBlockedReason(mid,names)`（两级混判）已删除、⚠ 不要再引回来；（b）`refilter()` 只按整机级过滤，商品级改由 `blockedPairs` 产出；（c）**第 2 步**写「另有 N 条上不了，机器保留、只跳过这几条：机器名 · 商品名（原因）」，**第 3 步**在被挡的商品行提前写明「⚠ N 台里有 M 台上不了这个商品（原因）· 提交时自动跳过」（同机型能上的商品行不带告警），预览与确认按钮按**条**扣减（「3 台 × 2 项 = 5 条（另有 1 条不支持，将跳过）」/「确认上架（3 台 · 跳过 1 条）」）；（d）`submit()` 跳过被挡组合（不占货道、不计成功条数），其余照常写入。连带三处：① 结果卡**单位按粒度分开**（成功＝台并带总条数、失败＝条，失败项逐条给「机器名 + 商品名 + 原因」，新增 `failUnit` / `okPairs` 两个字段）；② **单台**上架卡**部分商品被拦时照常出写卡**（只有全部商品都被拦才给说明卡），说明卡标题按粒度分两套（商品级「这个商品在这台机器上不了」/ 整机级「这台机器上架不了」），可执行项数按能上的算（按钮「确认上架（1 项）」）；③ **批量场景 P1 商品弹层不再置灰商品**（机器是客户挑好的，置灰＝替客户砍掉其余机器上的同一商品），单台场景仍置灰。</t>
         </is>
       </c>
       <c r="D34" s="5" t="inlineStr">
         <is>
-          <t>AiChat/api.js:9-13（chat/v2 SSE 与 ca-api 交互）；cardRegistry.js:12-23（现有 10 个能力卡片）</t>
-        </is>
-      </c>
-      <c r="E34" s="12" t="inlineStr">
-        <is>
-          <t>① 接口契约（请求 / 响应 / 错误码）随需求一并冻结，作为联调交付物；② 联调前先用 mock 契约跑通前端卡片；③ 核对不到的部分登记进 §12.2 待确认，不写进卡片文案｜影响：B7 配套能力与 mp_kb 结构无法在代码层核实</t>
+          <t>产品反馈 2026-10-28（用户原话，推翻 #25 的商品级部分）；需求说明 §5.1 / §5.2 / §5.6 / §12.1 定稿 #26；卡片设计稿 W2-b / W2-c；冒烟 MP 214 / PC 190（W2-j：机器保留在范围内不整台剔除、提示写明「机器保留、只跳过这几条」、第 3 步「2 台里有 1 台上不了这个商品」、能上的商品行不带告警、预览按条扣减、确认按钮带「跳过 1 条」、结果卡成功按台带总条数且失败按条并按「机器 · 商品」列出、数据校验被跳过商品没写进该机而同机其它商品照常写入、单台部分商品被拦照常出写卡、P1 单台商品级仍置灰而批量不置灰）</t>
+        </is>
+      </c>
+      <c r="E34" s="5" t="inlineStr">
+        <is>
+          <t>已落定，无未决风险</t>
         </is>
       </c>
     </row>
     <row r="35" ht="62" customHeight="1">
       <c r="A35" s="11" t="inlineStr">
         <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="B35" s="12" t="inlineStr">
+        <is>
+          <t>ca-api 不在代码库（盲区）</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>B7（NLU 泛化 + 机器点名 / 上下文）与 mp_kb 知识库结构无法在代码层面核对，只能核对到数据源与前端卡片缺口；需 ca-api 侧另行确认</t>
+        </is>
+      </c>
+      <c r="D35" s="5" t="inlineStr">
+        <is>
+          <t>AiChat/api.js:9-13（chat/v2 SSE 与 ca-api 交互）；cardRegistry.js:12-23（现有 10 个能力卡片）</t>
+        </is>
+      </c>
+      <c r="E35" s="12" t="inlineStr">
+        <is>
+          <t>① 接口契约（请求 / 响应 / 错误码）随需求一并冻结，作为联调交付物；② 联调前先用 mock 契约跑通前端卡片；③ 核对不到的部分登记进 §12.2 待确认，不写进卡片文案｜影响：B7 配套能力与 mp_kb 结构无法在代码层核实</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="62" customHeight="1">
+      <c r="A36" s="11" t="inlineStr">
+        <is>
           <t>R2</t>
         </is>
       </c>
-      <c r="B35" s="12" t="inlineStr">
+      <c r="B36" s="12" t="inlineStr">
         <is>
           <t>多台循环上架的部分失败反馈</t>
         </is>
       </c>
-      <c r="C35" s="5" t="inlineStr">
+      <c r="C36" s="5" t="inlineStr">
         <is>
           <t>单机循环时若部分机器被后台校验拦截（不支持机型 / 未绑定商品 code），需逐台列出失败机器与原因，不得整批报失败</t>
         </is>
       </c>
-      <c r="D35" s="5" t="inlineStr">
+      <c r="D36" s="5" t="inlineStr">
         <is>
           <t>与落定口径 1、2 配套，属前端卡片与 ca-api 交互约定</t>
         </is>
       </c>
-      <c r="E35" s="12" t="inlineStr">
+      <c r="E36" s="12" t="inlineStr">
         <is>
           <t>① 结果卡数据模型固定为 {succ[], fail[{机器, 原因}]}，成功 + 失败 = 命中总数；② 后端按机器维度返回错误码，前端原样透传、不改写；③ 重试只对 fail 项重新签发 confirm_id｜影响：批量上下架的结果展示与重试</t>
         </is>

</xml_diff>

<commit_message>
Publish index.html @ 2026-10-29 09:49:47
</commit_message>
<xml_diff>
--- a/iter.xlsx
+++ b/iter.xlsx
@@ -1340,7 +1340,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E36"/>
+  <dimension ref="A1:E37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="5" customWidth="1" min="1" max="1"/>
@@ -2050,7 +2050,7 @@
       </c>
       <c r="D27" s="5" t="inlineStr">
         <is>
-          <t>产品反馈 2026-10-28（附原型截图）；需求说明 §4.1 / §4.4 / §5.2 / §9.2 / §12.1 定稿 #19；卡片设计稿 W2-a / W2-b / W2-c（三个界面态）；冒烟 MP 191 / PC 184（W2 相关：第 1 步无机器选择区、步骤条 3 段仅 1 段激活、逐步进入第 2 / 3 步、第 3 步按机型分组（3 台两机型只出 2 块、块头「N 台 · 统一设置」、行数＝机型数 × 商品数）、智能柜默认「第 1 层」、售货机默认形如「A1 货道」、点位置 chip 呼出弹层并回填、确认按钮只在第 3 步；W2-d：直接进第 3 步、位置全锁 A1 货道、多台售货机合成 1 块、跳过智能柜）</t>
+          <t>产品反馈 2026-10-28（附原型截图）；需求说明 §4.1 / §4.4 / §5.2 / §9.2 / §12.1 定稿 #19；卡片设计稿 W2-a / W2-b / W2-c（三个界面态）；冒烟 MP 215 / PC 191（W2 相关：第 1 步无机器选择区、步骤条 3 段仅 1 段激活、步骤条第 3 段文案＝「上架」、逐步进入第 2 / 3 步、第 3 步按机型分组（3 台两机型只出 2 块、块头「N 台 · 统一设置」、行数＝机型数 × 商品数）、智能柜默认「第 1 层」、售货机默认形如「A1 货道」、点位置 chip 呼出弹层并回填、确认按钮只在第 3 步；W2-d：直接进第 3 步、位置全锁 A1 货道、多台售货机合成 1 块、跳过智能柜）</t>
         </is>
       </c>
       <c r="E27" s="5" t="inlineStr">
@@ -2249,55 +2249,82 @@
         </is>
       </c>
     </row>
-    <row r="35" ht="62" customHeight="1">
-      <c r="A35" s="11" t="inlineStr">
-        <is>
-          <t>R1</t>
-        </is>
-      </c>
-      <c r="B35" s="12" t="inlineStr">
-        <is>
-          <t>ca-api 不在代码库（盲区）</t>
+    <row r="35" ht="174" customHeight="1">
+      <c r="A35" s="4" t="inlineStr">
+        <is>
+          <t>33</t>
+        </is>
+      </c>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>批量上架步骤条第 3 段文案缩短（W2-a·b·c · 定稿 #27）</t>
         </is>
       </c>
       <c r="C35" s="5" t="inlineStr">
         <is>
-          <t>B7（NLU 泛化 + 机器点名 / 上下文）与 mp_kb 知识库结构无法在代码层面核对，只能核对到数据源与前端卡片缺口；需 ca-api 侧另行确认</t>
+          <t>2026-10-29 产品反馈（原话「批量上架商品的第三步字数减少一点，六个字加符号太多了；直接展示上架就行了」，附真机截图并用红框标出步骤条第 3 段）：原「位置 / 价格 / 库存」六个字 + 两个分隔符在手机上挤成两行，与「1 选商品」「2 选机器」四字严重不对称（步骤条三格是 flex:1 三等分，字越长越挤）。**改为「3 上架」**，三格宽度回到均匀。⚠ 只改**标题文案**——第 3 步的内容与列头不变（商品 / 位置或层 / 价格 / 库存，按机型一行统一设置，见 #27 / #28）。连带：第 2 步「下一步：位置 / 价格」→「下一步：上架」，与第 3 步标题对齐。两端共用同一份 `cardBatchOnshelf`，改一处两端同时生效。</t>
         </is>
       </c>
       <c r="D35" s="5" t="inlineStr">
         <is>
-          <t>AiChat/api.js:9-13（chat/v2 SSE 与 ca-api 交互）；cardRegistry.js:12-23（现有 10 个能力卡片）</t>
-        </is>
-      </c>
-      <c r="E35" s="12" t="inlineStr">
-        <is>
-          <t>① 接口契约（请求 / 响应 / 错误码）随需求一并冻结，作为联调交付物；② 联调前先用 mock 契约跑通前端卡片；③ 核对不到的部分登记进 §12.2 待确认，不写进卡片文案｜影响：B7 配套能力与 mp_kb 结构无法在代码层核实</t>
+          <t>产品反馈 2026-10-29（附真机截图）；需求说明 §5.2 / §12.1 定稿 #27；卡片设计稿 W2-a / W2-b / W2-c（三个界面态的步骤条与按钮同步）；冒烟 MP 215 / PC 191（步骤条第 3 段 textContent 归一化后 ===「3上架」、且 `.steps` 内不出现「位置 / 价格」）</t>
+        </is>
+      </c>
+      <c r="E35" s="5" t="inlineStr">
+        <is>
+          <t>已落定，无未决风险</t>
         </is>
       </c>
     </row>
     <row r="36" ht="62" customHeight="1">
       <c r="A36" s="11" t="inlineStr">
         <is>
+          <t>R1</t>
+        </is>
+      </c>
+      <c r="B36" s="12" t="inlineStr">
+        <is>
+          <t>ca-api 不在代码库（盲区）</t>
+        </is>
+      </c>
+      <c r="C36" s="5" t="inlineStr">
+        <is>
+          <t>B7（NLU 泛化 + 机器点名 / 上下文）与 mp_kb 知识库结构无法在代码层面核对，只能核对到数据源与前端卡片缺口；需 ca-api 侧另行确认</t>
+        </is>
+      </c>
+      <c r="D36" s="5" t="inlineStr">
+        <is>
+          <t>AiChat/api.js:9-13（chat/v2 SSE 与 ca-api 交互）；cardRegistry.js:12-23（现有 10 个能力卡片）</t>
+        </is>
+      </c>
+      <c r="E36" s="12" t="inlineStr">
+        <is>
+          <t>① 接口契约（请求 / 响应 / 错误码）随需求一并冻结，作为联调交付物；② 联调前先用 mock 契约跑通前端卡片；③ 核对不到的部分登记进 §12.2 待确认，不写进卡片文案｜影响：B7 配套能力与 mp_kb 结构无法在代码层核实</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="62" customHeight="1">
+      <c r="A37" s="11" t="inlineStr">
+        <is>
           <t>R2</t>
         </is>
       </c>
-      <c r="B36" s="12" t="inlineStr">
+      <c r="B37" s="12" t="inlineStr">
         <is>
           <t>多台循环上架的部分失败反馈</t>
         </is>
       </c>
-      <c r="C36" s="5" t="inlineStr">
+      <c r="C37" s="5" t="inlineStr">
         <is>
           <t>单机循环时若部分机器被后台校验拦截（不支持机型 / 未绑定商品 code），需逐台列出失败机器与原因，不得整批报失败</t>
         </is>
       </c>
-      <c r="D36" s="5" t="inlineStr">
+      <c r="D37" s="5" t="inlineStr">
         <is>
           <t>与落定口径 1、2 配套，属前端卡片与 ca-api 交互约定</t>
         </is>
       </c>
-      <c r="E36" s="12" t="inlineStr">
+      <c r="E37" s="12" t="inlineStr">
         <is>
           <t>① 结果卡数据模型固定为 {succ[], fail[{机器, 原因}]}，成功 + 失败 = 命中总数；② 后端按机器维度返回错误码，前端原样透传、不改写；③ 重试只对 fail 项重新签发 confirm_id｜影响：批量上下架的结果展示与重试</t>
         </is>

</xml_diff>